<commit_message>
Hermes: stock sync from rb-bot.xlsx
</commit_message>
<xml_diff>
--- a/tma_static/data/Roastberry_Прайс_2026.xlsx
+++ b/tma_static/data/Roastberry_Прайс_2026.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прайс 2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Прайс 2026" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1473,73 +1473,73 @@
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>🆕 моносорт</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>Вьетнам Блю Шонла</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="inlineStr">
-        <is>
-          <t>F E</t>
-        </is>
-      </c>
-      <c r="D29" s="12" t="n">
-        <v>2135</v>
-      </c>
-      <c r="E29" s="12" t="n">
-        <v>1925</v>
-      </c>
-      <c r="F29" s="12" t="n">
-        <v>1710</v>
-      </c>
-      <c r="G29" s="12" t="n">
-        <v>455</v>
-      </c>
-      <c r="H29" s="12" t="n">
-        <v>409.5</v>
-      </c>
-      <c r="I29" s="12" t="n">
-        <v>364</v>
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BLACK</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>Колумбия Клаудиа Колменарес Гейша мытый</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E29" s="15" t="n">
+        <v>3150</v>
+      </c>
+      <c r="F29" s="15" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G29" s="15" t="n">
+        <v>780</v>
+      </c>
+      <c r="H29" s="15" t="n">
+        <v>702</v>
+      </c>
+      <c r="I29" s="15" t="n">
+        <v>625</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>🆕 моносорт</t>
-        </is>
-      </c>
-      <c r="B30" s="10" t="inlineStr">
-        <is>
-          <t>Коста-Рика Тарразу мытый</t>
-        </is>
-      </c>
-      <c r="C30" s="11" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D30" s="12" t="n">
-        <v>2250</v>
-      </c>
-      <c r="E30" s="12" t="n">
-        <v>2025</v>
-      </c>
-      <c r="F30" s="12" t="n">
-        <v>1800</v>
-      </c>
-      <c r="G30" s="12" t="n">
-        <v>480</v>
-      </c>
-      <c r="H30" s="12" t="n">
-        <v>432</v>
-      </c>
-      <c r="I30" s="12" t="n">
-        <v>384</v>
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BLACK</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Эфиопия Иргач Адада гр.1 сухой</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>2390</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>2155</v>
+      </c>
+      <c r="F30" s="15" t="n">
+        <v>1915</v>
+      </c>
+      <c r="G30" s="15" t="n">
+        <v>560</v>
+      </c>
+      <c r="H30" s="15" t="n">
+        <v>504</v>
+      </c>
+      <c r="I30" s="15" t="n">
+        <v>450</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
@@ -1550,7 +1550,7 @@
       </c>
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>Колумбия Клаудиа Колменарес Гейша мытый</t>
+          <t>Эфиопия Иргач Билоя гр.2 сухой</t>
         </is>
       </c>
       <c r="C31" s="14" t="inlineStr">
@@ -1559,22 +1559,22 @@
         </is>
       </c>
       <c r="D31" s="15" t="n">
-        <v>3500</v>
+        <v>2232.5</v>
       </c>
       <c r="E31" s="15" t="n">
-        <v>3150</v>
+        <v>2010</v>
       </c>
       <c r="F31" s="15" t="n">
-        <v>2800</v>
+        <v>1790</v>
       </c>
       <c r="G31" s="15" t="n">
-        <v>780</v>
+        <v>525</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>702</v>
+        <v>472.5</v>
       </c>
       <c r="I31" s="15" t="n">
-        <v>625</v>
+        <v>420</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>Эфиопия Иргач Адада гр.1 сухой</t>
+          <t>Эфиопия Челчеле гр.1 сухой</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
@@ -1594,22 +1594,22 @@
         </is>
       </c>
       <c r="D32" s="15" t="n">
-        <v>2390</v>
+        <v>2862.5</v>
       </c>
       <c r="E32" s="15" t="n">
-        <v>2155</v>
+        <v>2580</v>
       </c>
       <c r="F32" s="15" t="n">
-        <v>1915</v>
+        <v>2290</v>
       </c>
       <c r="G32" s="15" t="n">
-        <v>560</v>
+        <v>655</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>504</v>
+        <v>589.5</v>
       </c>
       <c r="I32" s="15" t="n">
-        <v>450</v>
+        <v>525</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="B33" s="13" t="inlineStr">
         <is>
-          <t>Эфиопия Иргач Билоя гр.2 сухой</t>
+          <t>Эфиопия Иргач Челелекту мытый гр.1</t>
         </is>
       </c>
       <c r="C33" s="14" t="inlineStr">
@@ -1629,33 +1629,33 @@
         </is>
       </c>
       <c r="D33" s="15" t="n">
-        <v>2232.5</v>
+        <v>2862.5</v>
       </c>
       <c r="E33" s="15" t="n">
-        <v>2010</v>
+        <v>2580</v>
       </c>
       <c r="F33" s="15" t="n">
-        <v>1790</v>
+        <v>2290</v>
       </c>
       <c r="G33" s="15" t="n">
+        <v>655</v>
+      </c>
+      <c r="H33" s="15" t="n">
+        <v>589.5</v>
+      </c>
+      <c r="I33" s="15" t="n">
         <v>525</v>
-      </c>
-      <c r="H33" s="15" t="n">
-        <v>472.5</v>
-      </c>
-      <c r="I33" s="15" t="n">
-        <v>420</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>микролот • BLACK</t>
+          <t>микролот • BORЩ</t>
         </is>
       </c>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>Эфиопия Челчеле гр.1 сухой</t>
+          <t>Колумбия Хайро Арсило сухой</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
@@ -1685,12 +1685,12 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>микролот • BLACK</t>
+          <t>микролот • BORЩ</t>
         </is>
       </c>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Эфиопия Иргач Челелекту мытый гр.1</t>
+          <t>Колумбия Гонзало Кормана Катура сухой</t>
         </is>
       </c>
       <c r="C35" s="14" t="inlineStr">
@@ -1699,22 +1699,22 @@
         </is>
       </c>
       <c r="D35" s="15" t="n">
-        <v>2862.5</v>
+        <v>3500</v>
       </c>
       <c r="E35" s="15" t="n">
-        <v>2580</v>
+        <v>3150</v>
       </c>
       <c r="F35" s="15" t="n">
-        <v>2290</v>
+        <v>2800</v>
       </c>
       <c r="G35" s="15" t="n">
-        <v>655</v>
+        <v>780</v>
       </c>
       <c r="H35" s="15" t="n">
-        <v>589.5</v>
+        <v>702</v>
       </c>
       <c r="I35" s="15" t="n">
-        <v>525</v>
+        <v>625</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>Колумбия Хайро Арсило сухой</t>
+          <t>Смесь Экваториальная</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr">
@@ -1734,22 +1734,22 @@
         </is>
       </c>
       <c r="D36" s="15" t="n">
-        <v>2862.5</v>
+        <v>3020</v>
       </c>
       <c r="E36" s="15" t="n">
-        <v>2580</v>
+        <v>2720</v>
       </c>
       <c r="F36" s="15" t="n">
-        <v>2290</v>
+        <v>2420</v>
       </c>
       <c r="G36" s="15" t="n">
-        <v>655</v>
+        <v>685</v>
       </c>
       <c r="H36" s="15" t="n">
-        <v>589.5</v>
+        <v>616.5</v>
       </c>
       <c r="I36" s="15" t="n">
-        <v>525</v>
+        <v>550</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="B37" s="13" t="inlineStr">
         <is>
-          <t>Колумбия Гонзало Кормана Катура сухой</t>
+          <t>Эфиопия Арича гр.1 сухой</t>
         </is>
       </c>
       <c r="C37" s="14" t="inlineStr">
@@ -1769,92 +1769,92 @@
         </is>
       </c>
       <c r="D37" s="15" t="n">
+        <v>3020</v>
+      </c>
+      <c r="E37" s="15" t="n">
+        <v>2720</v>
+      </c>
+      <c r="F37" s="15" t="n">
+        <v>2420</v>
+      </c>
+      <c r="G37" s="15" t="n">
+        <v>685</v>
+      </c>
+      <c r="H37" s="15" t="n">
+        <v>616.5</v>
+      </c>
+      <c r="I37" s="15" t="n">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>🆕 микролот • BORЩ</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Бразилия SL28 Хани анаэроб.</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="n">
         <v>3500</v>
       </c>
-      <c r="E37" s="15" t="n">
+      <c r="E38" s="12" t="n">
         <v>3150</v>
       </c>
-      <c r="F37" s="15" t="n">
+      <c r="F38" s="12" t="n">
         <v>2800</v>
       </c>
-      <c r="G37" s="15" t="n">
+      <c r="G38" s="12" t="n">
         <v>780</v>
       </c>
-      <c r="H37" s="15" t="n">
+      <c r="H38" s="12" t="n">
         <v>702</v>
       </c>
-      <c r="I37" s="15" t="n">
+      <c r="I38" s="12" t="n">
         <v>625</v>
       </c>
     </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="13" t="inlineStr">
-        <is>
-          <t>микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>Смесь Экваториальная</t>
-        </is>
-      </c>
-      <c r="C38" s="14" t="inlineStr">
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>🆕 микролот • BORЩ</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Бразилия Судан Руме анаэроб.</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D38" s="15" t="n">
-        <v>3020</v>
-      </c>
-      <c r="E38" s="15" t="n">
-        <v>2720</v>
-      </c>
-      <c r="F38" s="15" t="n">
-        <v>2420</v>
-      </c>
-      <c r="G38" s="15" t="n">
-        <v>685</v>
-      </c>
-      <c r="H38" s="15" t="n">
-        <v>616.5</v>
-      </c>
-      <c r="I38" s="15" t="n">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="13" t="inlineStr">
-        <is>
-          <t>микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>Эфиопия Арича гр.1 сухой</t>
-        </is>
-      </c>
-      <c r="C39" s="14" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D39" s="15" t="n">
-        <v>3020</v>
-      </c>
-      <c r="E39" s="15" t="n">
-        <v>2720</v>
-      </c>
-      <c r="F39" s="15" t="n">
-        <v>2420</v>
-      </c>
-      <c r="G39" s="15" t="n">
-        <v>685</v>
-      </c>
-      <c r="H39" s="15" t="n">
-        <v>616.5</v>
-      </c>
-      <c r="I39" s="15" t="n">
-        <v>550</v>
+      <c r="D39" s="12" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E39" s="12" t="n">
+        <v>3150</v>
+      </c>
+      <c r="F39" s="12" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G39" s="12" t="n">
+        <v>780</v>
+      </c>
+      <c r="H39" s="12" t="n">
+        <v>702</v>
+      </c>
+      <c r="I39" s="12" t="n">
+        <v>625</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
@@ -1865,7 +1865,7 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Бразилия SL28 Хани анаэроб.</t>
+          <t>Бразилия Фазенда Лагуинья мундо анаэроб.</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
@@ -1893,73 +1893,65 @@
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>🆕 микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t>Бразилия Судан Руме анаэроб.</t>
-        </is>
-      </c>
-      <c r="C41" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D41" s="12" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E41" s="12" t="n">
-        <v>3150</v>
-      </c>
-      <c r="F41" s="12" t="n">
-        <v>2800</v>
-      </c>
-      <c r="G41" s="12" t="n">
-        <v>780</v>
-      </c>
-      <c r="H41" s="12" t="n">
-        <v>702</v>
-      </c>
-      <c r="I41" s="12" t="n">
-        <v>625</v>
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>микролот</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Колумбия Лили Роза Варгас Морено Чирозо Катуа </t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr"/>
+      <c r="D41" s="15" t="n">
+        <v>3102.5</v>
+      </c>
+      <c r="E41" s="15" t="n">
+        <v>2795</v>
+      </c>
+      <c r="F41" s="15" t="n">
+        <v>2485</v>
+      </c>
+      <c r="G41" s="15" t="n">
+        <v>700</v>
+      </c>
+      <c r="H41" s="15" t="n">
+        <v>630</v>
+      </c>
+      <c r="I41" s="15" t="n">
+        <v>560</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="10" t="inlineStr">
-        <is>
-          <t>🆕 микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B42" s="10" t="inlineStr">
-        <is>
-          <t>Бразилия Фазенда Лагуинья мундо анаэроб.</t>
-        </is>
-      </c>
-      <c r="C42" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D42" s="12" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E42" s="12" t="n">
-        <v>3150</v>
-      </c>
-      <c r="F42" s="12" t="n">
-        <v>2800</v>
-      </c>
-      <c r="G42" s="12" t="n">
-        <v>780</v>
-      </c>
-      <c r="H42" s="12" t="n">
-        <v>702</v>
-      </c>
-      <c r="I42" s="12" t="n">
-        <v>625</v>
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>микролот</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>Колумбия Хиросос мытый</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr"/>
+      <c r="D42" s="15" t="n">
+        <v>2547.5</v>
+      </c>
+      <c r="E42" s="15" t="n">
+        <v>2295</v>
+      </c>
+      <c r="F42" s="15" t="n">
+        <v>2040</v>
+      </c>
+      <c r="G42" s="15" t="n">
+        <v>590</v>
+      </c>
+      <c r="H42" s="15" t="n">
+        <v>531</v>
+      </c>
+      <c r="I42" s="15" t="n">
+        <v>475</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
@@ -1970,27 +1962,27 @@
       </c>
       <c r="B43" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Колумбия Лили Роза Варгас Морено Чирозо Катуа </t>
+          <t>Руанада Нямашеки хилс сухой</t>
         </is>
       </c>
       <c r="C43" s="14" t="inlineStr"/>
       <c r="D43" s="15" t="n">
-        <v>3102.5</v>
+        <v>2862.5</v>
       </c>
       <c r="E43" s="15" t="n">
-        <v>2795</v>
+        <v>2580</v>
       </c>
       <c r="F43" s="15" t="n">
-        <v>2485</v>
+        <v>2290</v>
       </c>
       <c r="G43" s="15" t="n">
-        <v>700</v>
+        <v>655</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>630</v>
+        <v>589.5</v>
       </c>
       <c r="I43" s="15" t="n">
-        <v>560</v>
+        <v>525</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
@@ -2001,89 +1993,97 @@
       </c>
       <c r="B44" s="13" t="inlineStr">
         <is>
-          <t>Колумбия Хиросос мытый</t>
+          <t>КолумбияХайро Асрило инфьюз Маракуйя</t>
         </is>
       </c>
       <c r="C44" s="14" t="inlineStr"/>
       <c r="D44" s="15" t="n">
-        <v>2547.5</v>
+        <v>4925</v>
       </c>
       <c r="E44" s="15" t="n">
-        <v>2295</v>
+        <v>4435</v>
       </c>
       <c r="F44" s="15" t="n">
-        <v>2040</v>
+        <v>3940</v>
       </c>
       <c r="G44" s="15" t="n">
-        <v>590</v>
+        <v>1065</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>531</v>
+        <v>958.5</v>
       </c>
       <c r="I44" s="15" t="n">
-        <v>475</v>
+        <v>855</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="13" t="inlineStr">
-        <is>
-          <t>микролот</t>
-        </is>
-      </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>Руанада Нямашеки хилс сухой</t>
-        </is>
-      </c>
-      <c r="C45" s="14" t="inlineStr"/>
-      <c r="D45" s="15" t="n">
-        <v>2862.5</v>
-      </c>
-      <c r="E45" s="15" t="n">
-        <v>2580</v>
-      </c>
-      <c r="F45" s="15" t="n">
-        <v>2290</v>
-      </c>
-      <c r="G45" s="15" t="n">
-        <v>655</v>
-      </c>
-      <c r="H45" s="15" t="n">
-        <v>589.5</v>
-      </c>
-      <c r="I45" s="15" t="n">
-        <v>525</v>
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>🆕 микролот</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>Колумбия Кастильо</t>
+        </is>
+      </c>
+      <c r="C45" s="11" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D45" s="12" t="n">
+        <v>2847.5</v>
+      </c>
+      <c r="E45" s="12" t="n">
+        <v>2565</v>
+      </c>
+      <c r="F45" s="12" t="n">
+        <v>2280</v>
+      </c>
+      <c r="G45" s="12" t="n">
+        <v>650</v>
+      </c>
+      <c r="H45" s="12" t="n">
+        <v>585</v>
+      </c>
+      <c r="I45" s="12" t="n">
+        <v>520</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="13" t="inlineStr">
-        <is>
-          <t>микролот</t>
-        </is>
-      </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>КолумбияХайро Асрило инфьюз Маракуйя</t>
-        </is>
-      </c>
-      <c r="C46" s="14" t="inlineStr"/>
-      <c r="D46" s="15" t="n">
-        <v>4925</v>
-      </c>
-      <c r="E46" s="15" t="n">
-        <v>4435</v>
-      </c>
-      <c r="F46" s="15" t="n">
-        <v>3940</v>
-      </c>
-      <c r="G46" s="15" t="n">
-        <v>1065</v>
-      </c>
-      <c r="H46" s="15" t="n">
-        <v>958.5</v>
-      </c>
-      <c r="I46" s="15" t="n">
-        <v>855</v>
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>🆕 микролот</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>Колумбия Пачамама</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D46" s="12" t="n">
+        <v>4842.5</v>
+      </c>
+      <c r="E46" s="12" t="n">
+        <v>4360</v>
+      </c>
+      <c r="F46" s="12" t="n">
+        <v>3875</v>
+      </c>
+      <c r="G46" s="12" t="n">
+        <v>1050</v>
+      </c>
+      <c r="H46" s="12" t="n">
+        <v>945</v>
+      </c>
+      <c r="I46" s="12" t="n">
+        <v>840</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
@@ -2094,7 +2094,7 @@
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>Колумбия Кастильо</t>
+          <t>Колумбия Маракуйя</t>
         </is>
       </c>
       <c r="C47" s="11" t="inlineStr">
@@ -2103,91 +2103,21 @@
         </is>
       </c>
       <c r="D47" s="12" t="n">
-        <v>2847.5</v>
+        <v>5922.5</v>
       </c>
       <c r="E47" s="12" t="n">
-        <v>2565</v>
+        <v>5335</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>2280</v>
+        <v>4740</v>
       </c>
       <c r="G47" s="12" t="n">
-        <v>650</v>
+        <v>1265</v>
       </c>
       <c r="H47" s="12" t="n">
-        <v>585</v>
+        <v>1138.5</v>
       </c>
       <c r="I47" s="12" t="n">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="10" t="inlineStr">
-        <is>
-          <t>🆕 микролот</t>
-        </is>
-      </c>
-      <c r="B48" s="10" t="inlineStr">
-        <is>
-          <t>Колумбия Пачамама</t>
-        </is>
-      </c>
-      <c r="C48" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D48" s="12" t="n">
-        <v>4842.5</v>
-      </c>
-      <c r="E48" s="12" t="n">
-        <v>4360</v>
-      </c>
-      <c r="F48" s="12" t="n">
-        <v>3875</v>
-      </c>
-      <c r="G48" s="12" t="n">
-        <v>1050</v>
-      </c>
-      <c r="H48" s="12" t="n">
-        <v>945</v>
-      </c>
-      <c r="I48" s="12" t="n">
-        <v>840</v>
-      </c>
-    </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="10" t="inlineStr">
-        <is>
-          <t>🆕 микролот</t>
-        </is>
-      </c>
-      <c r="B49" s="10" t="inlineStr">
-        <is>
-          <t>Колумбия Маракуйя</t>
-        </is>
-      </c>
-      <c r="C49" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D49" s="12" t="n">
-        <v>5922.5</v>
-      </c>
-      <c r="E49" s="12" t="n">
-        <v>5335</v>
-      </c>
-      <c r="F49" s="12" t="n">
-        <v>4740</v>
-      </c>
-      <c r="G49" s="12" t="n">
-        <v>1265</v>
-      </c>
-      <c r="H49" s="12" t="n">
-        <v>1138.5</v>
-      </c>
-      <c r="I49" s="12" t="n">
         <v>1015</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Bishop: Auto stock sync from 1C: stock updates 25
</commit_message>
<xml_diff>
--- a/tma_static/data/Roastberry_Прайс_2026.xlsx
+++ b/tma_static/data/Roastberry_Прайс_2026.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1543,38 +1543,38 @@
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="13" t="inlineStr">
-        <is>
-          <t>микролот • BLACK</t>
-        </is>
-      </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>Колумбия Клаудиа Колменарес Гейша мытый</t>
-        </is>
-      </c>
-      <c r="C31" s="14" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D31" s="15" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E31" s="15" t="n">
-        <v>3150</v>
-      </c>
-      <c r="F31" s="15" t="n">
-        <v>2800</v>
-      </c>
-      <c r="G31" s="15" t="n">
-        <v>780</v>
-      </c>
-      <c r="H31" s="15" t="n">
-        <v>702</v>
-      </c>
-      <c r="I31" s="15" t="n">
-        <v>625</v>
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>🆕 моносорт</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Гватемалла Грок</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>F E</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="n">
+        <v>2120</v>
+      </c>
+      <c r="E31" s="12" t="n">
+        <v>1910</v>
+      </c>
+      <c r="F31" s="12" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G31" s="12" t="n">
+        <v>455</v>
+      </c>
+      <c r="H31" s="12" t="n">
+        <v>409.5</v>
+      </c>
+      <c r="I31" s="12" t="n">
+        <v>364</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>Эфиопия Иргач Адада гр.1 сухой</t>
+          <t>Колумбия Клаудиа Колменарес Гейша мытый</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
@@ -1594,22 +1594,22 @@
         </is>
       </c>
       <c r="D32" s="15" t="n">
-        <v>2390</v>
+        <v>3500</v>
       </c>
       <c r="E32" s="15" t="n">
-        <v>2155</v>
+        <v>3150</v>
       </c>
       <c r="F32" s="15" t="n">
-        <v>1915</v>
+        <v>2800</v>
       </c>
       <c r="G32" s="15" t="n">
-        <v>560</v>
+        <v>780</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>504</v>
+        <v>702</v>
       </c>
       <c r="I32" s="15" t="n">
-        <v>450</v>
+        <v>625</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="B33" s="13" t="inlineStr">
         <is>
-          <t>Эфиопия Иргач Билоя гр.2 сухой</t>
+          <t>Эфиопия Иргач Адада гр.1 сухой</t>
         </is>
       </c>
       <c r="C33" s="14" t="inlineStr">
@@ -1629,22 +1629,22 @@
         </is>
       </c>
       <c r="D33" s="15" t="n">
-        <v>2232.5</v>
+        <v>2390</v>
       </c>
       <c r="E33" s="15" t="n">
-        <v>2010</v>
+        <v>2155</v>
       </c>
       <c r="F33" s="15" t="n">
-        <v>1790</v>
+        <v>1915</v>
       </c>
       <c r="G33" s="15" t="n">
-        <v>525</v>
+        <v>560</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>472.5</v>
+        <v>504</v>
       </c>
       <c r="I33" s="15" t="n">
-        <v>420</v>
+        <v>450</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>Эфиопия Челчеле гр.1 сухой</t>
+          <t>Эфиопия Иргач Билоя гр.2 сухой</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
@@ -1664,22 +1664,22 @@
         </is>
       </c>
       <c r="D34" s="15" t="n">
-        <v>2862.5</v>
+        <v>2232.5</v>
       </c>
       <c r="E34" s="15" t="n">
-        <v>2580</v>
+        <v>2010</v>
       </c>
       <c r="F34" s="15" t="n">
-        <v>2290</v>
+        <v>1790</v>
       </c>
       <c r="G34" s="15" t="n">
-        <v>655</v>
+        <v>525</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>589.5</v>
+        <v>472.5</v>
       </c>
       <c r="I34" s="15" t="n">
-        <v>525</v>
+        <v>420</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Эфиопия Иргач Челелекту мытый гр.1</t>
+          <t>Эфиопия Челчеле гр.1 сухой</t>
         </is>
       </c>
       <c r="C35" s="14" t="inlineStr">
@@ -1720,12 +1720,12 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>микролот • BORЩ</t>
+          <t>микролот • BLACK</t>
         </is>
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>Колумбия Хайро Арсило сухой</t>
+          <t>Эфиопия Иргач Челелекту мытый гр.1</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="B37" s="13" t="inlineStr">
         <is>
-          <t>Колумбия Гонзало Кормана Катура сухой</t>
+          <t>Колумбия Хайро Арсило сухой</t>
         </is>
       </c>
       <c r="C37" s="14" t="inlineStr">
@@ -1769,22 +1769,22 @@
         </is>
       </c>
       <c r="D37" s="15" t="n">
-        <v>3500</v>
+        <v>2862.5</v>
       </c>
       <c r="E37" s="15" t="n">
-        <v>3150</v>
+        <v>2580</v>
       </c>
       <c r="F37" s="15" t="n">
-        <v>2800</v>
+        <v>2290</v>
       </c>
       <c r="G37" s="15" t="n">
-        <v>780</v>
+        <v>655</v>
       </c>
       <c r="H37" s="15" t="n">
-        <v>702</v>
+        <v>589.5</v>
       </c>
       <c r="I37" s="15" t="n">
-        <v>625</v>
+        <v>525</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>Смесь Экваториальная</t>
+          <t>Колумбия Гонзало Кормана Катура сухой</t>
         </is>
       </c>
       <c r="C38" s="14" t="inlineStr">
@@ -1804,22 +1804,22 @@
         </is>
       </c>
       <c r="D38" s="15" t="n">
-        <v>3020</v>
+        <v>3500</v>
       </c>
       <c r="E38" s="15" t="n">
-        <v>2720</v>
+        <v>3150</v>
       </c>
       <c r="F38" s="15" t="n">
-        <v>2420</v>
+        <v>2800</v>
       </c>
       <c r="G38" s="15" t="n">
-        <v>685</v>
+        <v>780</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>616.5</v>
+        <v>702</v>
       </c>
       <c r="I38" s="15" t="n">
-        <v>550</v>
+        <v>625</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="B39" s="13" t="inlineStr">
         <is>
-          <t>Эфиопия Арича гр.1 сухой</t>
+          <t>Смесь Экваториальная</t>
         </is>
       </c>
       <c r="C39" s="14" t="inlineStr">
@@ -1858,38 +1858,38 @@
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t>🆕 микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B40" s="10" t="inlineStr">
-        <is>
-          <t>Бразилия SL28 Хани анаэроб.</t>
-        </is>
-      </c>
-      <c r="C40" s="11" t="inlineStr">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BORЩ</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>Эфиопия Арича гр.1 сухой</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D40" s="12" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E40" s="12" t="n">
-        <v>3150</v>
-      </c>
-      <c r="F40" s="12" t="n">
-        <v>2800</v>
-      </c>
-      <c r="G40" s="12" t="n">
-        <v>780</v>
-      </c>
-      <c r="H40" s="12" t="n">
-        <v>702</v>
-      </c>
-      <c r="I40" s="12" t="n">
-        <v>625</v>
+      <c r="D40" s="15" t="n">
+        <v>3020</v>
+      </c>
+      <c r="E40" s="15" t="n">
+        <v>2720</v>
+      </c>
+      <c r="F40" s="15" t="n">
+        <v>2420</v>
+      </c>
+      <c r="G40" s="15" t="n">
+        <v>685</v>
+      </c>
+      <c r="H40" s="15" t="n">
+        <v>616.5</v>
+      </c>
+      <c r="I40" s="15" t="n">
+        <v>550</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Бразилия Судан Руме анаэроб.</t>
+          <t>Бразилия SL28 Хани анаэроб.</t>
         </is>
       </c>
       <c r="C41" s="11" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Бразилия Фазенда Лагуинья мундо анаэроб.</t>
+          <t>Бразилия Судан Руме анаэроб.</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
@@ -1963,34 +1963,38 @@
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="13" t="inlineStr">
-        <is>
-          <t>микролот</t>
-        </is>
-      </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Колумбия Лили Роза Варгас Морено Чирозо Катуа </t>
-        </is>
-      </c>
-      <c r="C43" s="14" t="inlineStr"/>
-      <c r="D43" s="15" t="n">
-        <v>3102.5</v>
-      </c>
-      <c r="E43" s="15" t="n">
-        <v>2795</v>
-      </c>
-      <c r="F43" s="15" t="n">
-        <v>2485</v>
-      </c>
-      <c r="G43" s="15" t="n">
-        <v>700</v>
-      </c>
-      <c r="H43" s="15" t="n">
-        <v>630</v>
-      </c>
-      <c r="I43" s="15" t="n">
-        <v>560</v>
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>🆕 микролот • BORЩ</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>Бразилия Фазенда Лагуинья мундо анаэроб.</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E43" s="12" t="n">
+        <v>3150</v>
+      </c>
+      <c r="F43" s="12" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G43" s="12" t="n">
+        <v>780</v>
+      </c>
+      <c r="H43" s="12" t="n">
+        <v>702</v>
+      </c>
+      <c r="I43" s="12" t="n">
+        <v>625</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
@@ -2001,27 +2005,27 @@
       </c>
       <c r="B44" s="13" t="inlineStr">
         <is>
-          <t>Колумбия Хиросос мытый</t>
+          <t xml:space="preserve">Колумбия Лили Роза Варгас Морено Чирозо Катуа </t>
         </is>
       </c>
       <c r="C44" s="14" t="inlineStr"/>
       <c r="D44" s="15" t="n">
-        <v>2547.5</v>
+        <v>3102.5</v>
       </c>
       <c r="E44" s="15" t="n">
-        <v>2295</v>
+        <v>2795</v>
       </c>
       <c r="F44" s="15" t="n">
-        <v>2040</v>
+        <v>2485</v>
       </c>
       <c r="G44" s="15" t="n">
-        <v>590</v>
+        <v>700</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>531</v>
+        <v>630</v>
       </c>
       <c r="I44" s="15" t="n">
-        <v>475</v>
+        <v>560</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
@@ -2032,27 +2036,27 @@
       </c>
       <c r="B45" s="13" t="inlineStr">
         <is>
-          <t>Руанада Нямашеки хилс сухой</t>
+          <t>Колумбия Хиросос мытый</t>
         </is>
       </c>
       <c r="C45" s="14" t="inlineStr"/>
       <c r="D45" s="15" t="n">
-        <v>2862.5</v>
+        <v>2547.5</v>
       </c>
       <c r="E45" s="15" t="n">
-        <v>2580</v>
+        <v>2295</v>
       </c>
       <c r="F45" s="15" t="n">
-        <v>2290</v>
+        <v>2040</v>
       </c>
       <c r="G45" s="15" t="n">
-        <v>655</v>
+        <v>590</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>589.5</v>
+        <v>531</v>
       </c>
       <c r="I45" s="15" t="n">
-        <v>525</v>
+        <v>475</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
@@ -2063,62 +2067,58 @@
       </c>
       <c r="B46" s="13" t="inlineStr">
         <is>
-          <t>КолумбияХайро Асрило инфьюз Маракуйя</t>
+          <t>Руанада Нямашеки хилс сухой</t>
         </is>
       </c>
       <c r="C46" s="14" t="inlineStr"/>
       <c r="D46" s="15" t="n">
+        <v>2862.5</v>
+      </c>
+      <c r="E46" s="15" t="n">
+        <v>2580</v>
+      </c>
+      <c r="F46" s="15" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G46" s="15" t="n">
+        <v>655</v>
+      </c>
+      <c r="H46" s="15" t="n">
+        <v>589.5</v>
+      </c>
+      <c r="I46" s="15" t="n">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>микролот</t>
+        </is>
+      </c>
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>КолумбияХайро Асрило инфьюз Маракуйя</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr"/>
+      <c r="D47" s="15" t="n">
         <v>4925</v>
       </c>
-      <c r="E46" s="15" t="n">
+      <c r="E47" s="15" t="n">
         <v>4435</v>
       </c>
-      <c r="F46" s="15" t="n">
+      <c r="F47" s="15" t="n">
         <v>3940</v>
       </c>
-      <c r="G46" s="15" t="n">
+      <c r="G47" s="15" t="n">
         <v>1065</v>
       </c>
-      <c r="H46" s="15" t="n">
+      <c r="H47" s="15" t="n">
         <v>958.5</v>
       </c>
-      <c r="I46" s="15" t="n">
+      <c r="I47" s="15" t="n">
         <v>855</v>
-      </c>
-    </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="10" t="inlineStr">
-        <is>
-          <t>🆕 микролот</t>
-        </is>
-      </c>
-      <c r="B47" s="10" t="inlineStr">
-        <is>
-          <t>Колумбия Кастильо</t>
-        </is>
-      </c>
-      <c r="C47" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D47" s="12" t="n">
-        <v>2847.5</v>
-      </c>
-      <c r="E47" s="12" t="n">
-        <v>2565</v>
-      </c>
-      <c r="F47" s="12" t="n">
-        <v>2280</v>
-      </c>
-      <c r="G47" s="12" t="n">
-        <v>650</v>
-      </c>
-      <c r="H47" s="12" t="n">
-        <v>585</v>
-      </c>
-      <c r="I47" s="12" t="n">
-        <v>520</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Колумбия Пачамама</t>
+          <t>Колумбия Кастильо</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
@@ -2138,22 +2138,22 @@
         </is>
       </c>
       <c r="D48" s="12" t="n">
-        <v>4842.5</v>
+        <v>2847.5</v>
       </c>
       <c r="E48" s="12" t="n">
-        <v>4360</v>
+        <v>2565</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3875</v>
+        <v>2280</v>
       </c>
       <c r="G48" s="12" t="n">
-        <v>1050</v>
+        <v>650</v>
       </c>
       <c r="H48" s="12" t="n">
-        <v>945</v>
+        <v>585</v>
       </c>
       <c r="I48" s="12" t="n">
-        <v>840</v>
+        <v>520</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
@@ -2164,30 +2164,65 @@
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
+          <t>Колумбия Пачамама</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D49" s="12" t="n">
+        <v>4842.5</v>
+      </c>
+      <c r="E49" s="12" t="n">
+        <v>4360</v>
+      </c>
+      <c r="F49" s="12" t="n">
+        <v>3875</v>
+      </c>
+      <c r="G49" s="12" t="n">
+        <v>1050</v>
+      </c>
+      <c r="H49" s="12" t="n">
+        <v>945</v>
+      </c>
+      <c r="I49" s="12" t="n">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>🆕 микролот</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
           <t>Колумбия Маракуйя</t>
         </is>
       </c>
-      <c r="C49" s="11" t="inlineStr">
+      <c r="C50" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D49" s="12" t="n">
+      <c r="D50" s="12" t="n">
         <v>5922.5</v>
       </c>
-      <c r="E49" s="12" t="n">
+      <c r="E50" s="12" t="n">
         <v>5335</v>
       </c>
-      <c r="F49" s="12" t="n">
+      <c r="F50" s="12" t="n">
         <v>4740</v>
       </c>
-      <c r="G49" s="12" t="n">
+      <c r="G50" s="12" t="n">
         <v>1265</v>
       </c>
-      <c r="H49" s="12" t="n">
+      <c r="H50" s="12" t="n">
         <v>1138.5</v>
       </c>
-      <c r="I49" s="12" t="n">
+      <c r="I50" s="12" t="n">
         <v>1015</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Bishop: Auto stock sync from 1C: stock updates 0
</commit_message>
<xml_diff>
--- a/tma_static/data/Roastberry_Прайс_2026.xlsx
+++ b/tma_static/data/Roastberry_Прайс_2026.xlsx
@@ -675,7 +675,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>ХАНИ</t>
+          <t>ВЕНЕЦИЯ</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>ВЕНЕЦИЯ</t>
+          <t>ХАНИ</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Бразилия Серрадо сухой/Бразилия Дарк </t>
+          <t>Бразилия САН РАФАЕЛЬ сухой</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -789,22 +789,22 @@
         </is>
       </c>
       <c r="D9" s="9" t="n">
-        <v>2015</v>
+        <v>2070</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>1815</v>
+        <v>1865</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>1615</v>
+        <v>1660</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>435</v>
+        <v>445</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>391.5</v>
+        <v>400.5</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>348</v>
+        <v>356</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -815,31 +815,31 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Бразилия САН РАФАЕЛЬ сухой</t>
+          <t>Бразилия Серрадо желтый бурбон сухой</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>2070</v>
+        <v>2120</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>1865</v>
+        <v>1910</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>1660</v>
+        <v>1700</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>445</v>
+        <v>455</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>400.5</v>
+        <v>409.5</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>356</v>
+        <v>364</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
@@ -850,101 +850,101 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Бразилия Серрадо желтый бурбон сухой</t>
+          <t xml:space="preserve">Бразилия Серрадо сухой/Бразилия Дарк </t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D11" s="9" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>1815</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>1615</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>435</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>391.5</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>🆕 моносорт</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Вьетнам Блю Шонла</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>F E</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="n">
+        <v>2135</v>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>1925</v>
+      </c>
+      <c r="F12" s="12" t="n">
+        <v>1710</v>
+      </c>
+      <c r="G12" s="12" t="n">
+        <v>455</v>
+      </c>
+      <c r="H12" s="12" t="n">
+        <v>409.5</v>
+      </c>
+      <c r="I12" s="12" t="n">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>🆕 моносорт</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Гватемалла Грок</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>F E</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="n">
         <v>2120</v>
       </c>
-      <c r="E11" s="9" t="n">
+      <c r="E13" s="12" t="n">
         <v>1910</v>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F13" s="12" t="n">
         <v>1700</v>
       </c>
-      <c r="G11" s="9" t="n">
+      <c r="G13" s="12" t="n">
         <v>455</v>
       </c>
-      <c r="H11" s="9" t="n">
+      <c r="H13" s="12" t="n">
         <v>409.5</v>
       </c>
-      <c r="I11" s="9" t="n">
+      <c r="I13" s="12" t="n">
         <v>364</v>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>моносорт</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Гватемалла Декаф</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="n">
-        <v>2440</v>
-      </c>
-      <c r="E12" s="9" t="n">
-        <v>2200</v>
-      </c>
-      <c r="F12" s="9" t="n">
-        <v>1955</v>
-      </c>
-      <c r="G12" s="9" t="n">
-        <v>520</v>
-      </c>
-      <c r="H12" s="9" t="n">
-        <v>468</v>
-      </c>
-      <c r="I12" s="9" t="n">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>моносорт</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Гондурас Сан Николас мытый</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="n">
-        <v>2175</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <v>1960</v>
-      </c>
-      <c r="F13" s="9" t="n">
-        <v>1740</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>465</v>
-      </c>
-      <c r="H13" s="9" t="n">
-        <v>418.5</v>
-      </c>
-      <c r="I13" s="9" t="n">
-        <v>372</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
@@ -955,31 +955,31 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Кения АА мытый</t>
+          <t>Гватемалла Декаф</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D14" s="9" t="n">
-        <v>2595</v>
+        <v>2440</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>2340</v>
+        <v>2200</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>2080</v>
+        <v>1955</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>550</v>
+        <v>520</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>495</v>
+        <v>468</v>
       </c>
       <c r="I14" s="9" t="n">
-        <v>440</v>
+        <v>416</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -990,31 +990,31 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Кения Центральный провинции АБ мытый</t>
+          <t>Гондурас Сан Николас мытый</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>E F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D15" s="9" t="n">
-        <v>2490</v>
+        <v>2175</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>2245</v>
+        <v>1960</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>1995</v>
+        <v>1740</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>530</v>
+        <v>465</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>477</v>
+        <v>418.5</v>
       </c>
       <c r="I15" s="9" t="n">
-        <v>424</v>
+        <v>372</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
@@ -1025,31 +1025,31 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Колумбия Андино мытый</t>
+          <t>Кения АА мытый</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>E F</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D16" s="9" t="n">
-        <v>2175</v>
+        <v>2595</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>1960</v>
+        <v>2340</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>1740</v>
+        <v>2080</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>465</v>
+        <v>550</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>418.5</v>
+        <v>495</v>
       </c>
       <c r="I16" s="9" t="n">
-        <v>372</v>
+        <v>440</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
@@ -1060,66 +1060,66 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Никарагуа Марагаджип мытый</t>
+          <t>Кения Центральный провинции АБ мытый</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>E F</t>
         </is>
       </c>
       <c r="D17" s="9" t="n">
-        <v>2545</v>
+        <v>2490</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>2295</v>
+        <v>2245</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>2040</v>
+        <v>1995</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>540</v>
+        <v>530</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>486</v>
+        <v>477</v>
       </c>
       <c r="I17" s="9" t="n">
-        <v>432</v>
+        <v>424</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>моносорт</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Перу Гр.1</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="n">
-        <v>2230</v>
-      </c>
-      <c r="E18" s="9" t="n">
-        <v>2010</v>
-      </c>
-      <c r="F18" s="9" t="n">
-        <v>1785</v>
-      </c>
-      <c r="G18" s="9" t="n">
-        <v>475</v>
-      </c>
-      <c r="H18" s="9" t="n">
-        <v>427.5</v>
-      </c>
-      <c r="I18" s="9" t="n">
-        <v>380</v>
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>🆕 моносорт</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Китай Симао Гр.1 мытый</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>F E</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>1815</v>
+      </c>
+      <c r="F18" s="12" t="n">
+        <v>1615</v>
+      </c>
+      <c r="G18" s="12" t="n">
+        <v>435</v>
+      </c>
+      <c r="H18" s="12" t="n">
+        <v>391.5</v>
+      </c>
+      <c r="I18" s="12" t="n">
+        <v>348</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
@@ -1130,66 +1130,66 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Перу Монте Верде сухой</t>
+          <t>Колумбия Андино мытый</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E F</t>
         </is>
       </c>
       <c r="D19" s="9" t="n">
-        <v>2620</v>
+        <v>2175</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>2360</v>
+        <v>1960</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>2100</v>
+        <v>1740</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>555</v>
+        <v>465</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>499.5</v>
+        <v>418.5</v>
       </c>
       <c r="I19" s="9" t="n">
-        <v>444</v>
+        <v>372</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>моносорт</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Руанада Мутителли 15+</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>2230</v>
-      </c>
-      <c r="E20" s="9" t="n">
-        <v>2010</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>1785</v>
-      </c>
-      <c r="G20" s="9" t="n">
-        <v>475</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>427.5</v>
-      </c>
-      <c r="I20" s="9" t="n">
-        <v>380</v>
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>🆕 моносорт</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Коста-Рика Тарразу мытый</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>2250</v>
+      </c>
+      <c r="E20" s="12" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F20" s="12" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G20" s="12" t="n">
+        <v>480</v>
+      </c>
+      <c r="H20" s="12" t="n">
+        <v>432</v>
+      </c>
+      <c r="I20" s="12" t="n">
+        <v>384</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
@@ -1200,31 +1200,31 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Танзания АА</t>
+          <t>Никарагуа Марагаджип мытый</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D21" s="9" t="n">
-        <v>2335</v>
+        <v>2545</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>2105</v>
+        <v>2295</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>1870</v>
+        <v>2040</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>495</v>
+        <v>540</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>445.5</v>
+        <v>486</v>
       </c>
       <c r="I21" s="9" t="n">
-        <v>396</v>
+        <v>432</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Уганда Рувензор сухой</t>
+          <t>Перу Гр.1</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
@@ -1244,22 +1244,22 @@
         </is>
       </c>
       <c r="D22" s="9" t="n">
-        <v>2015</v>
+        <v>2230</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>1815</v>
+        <v>2010</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>1615</v>
+        <v>1785</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>435</v>
+        <v>475</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>391.5</v>
+        <v>427.5</v>
       </c>
       <c r="I22" s="9" t="n">
-        <v>348</v>
+        <v>380</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
@@ -1270,31 +1270,31 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Уганда Вугар Элгон мытый </t>
+          <t>Перу Монте Верде сухой</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D23" s="9" t="n">
-        <v>2070</v>
+        <v>2620</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>1865</v>
+        <v>2360</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>1660</v>
+        <v>2100</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>445</v>
+        <v>555</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>400.5</v>
+        <v>499.5</v>
       </c>
       <c r="I23" s="9" t="n">
-        <v>356</v>
+        <v>444</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
@@ -1305,31 +1305,31 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Эфиопия Арича Гр.3 сухой </t>
+          <t>Руанада Мутителли 15+</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D24" s="9" t="n">
-        <v>2175</v>
+        <v>2230</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>1960</v>
+        <v>2010</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>1740</v>
+        <v>1785</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>465</v>
+        <v>475</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>418.5</v>
+        <v>427.5</v>
       </c>
       <c r="I24" s="9" t="n">
-        <v>372</v>
+        <v>380</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
@@ -1340,31 +1340,31 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Эфиопия Иргач Гр.4 ТОП сухой /Эфиопи Милк (темн)</t>
+          <t>Танзания АА</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D25" s="9" t="n">
-        <v>2015</v>
+        <v>2335</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>1815</v>
+        <v>2105</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>1615</v>
+        <v>1870</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>435</v>
+        <v>495</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>391.5</v>
+        <v>445.5</v>
       </c>
       <c r="I25" s="9" t="n">
-        <v>348</v>
+        <v>396</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
@@ -1375,31 +1375,31 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Эфиопия Лиму Гр.2 мытый</t>
+          <t xml:space="preserve">Уганда Вугар Элгон мытый </t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D26" s="9" t="n">
-        <v>2120</v>
+        <v>2070</v>
       </c>
       <c r="E26" s="9" t="n">
-        <v>1910</v>
+        <v>1865</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>1700</v>
+        <v>1660</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>455</v>
+        <v>445</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>409.5</v>
+        <v>400.5</v>
       </c>
       <c r="I26" s="9" t="n">
-        <v>364</v>
+        <v>356</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
@@ -1410,170 +1410,170 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
+          <t>Уганда Рувензор сухой</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>1815</v>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>1615</v>
+      </c>
+      <c r="G27" s="9" t="n">
+        <v>435</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>391.5</v>
+      </c>
+      <c r="I27" s="9" t="n">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>моносорт</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Эфиопия Арича Гр.3 сухой </t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>2175</v>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>1960</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>1740</v>
+      </c>
+      <c r="G28" s="9" t="n">
+        <v>465</v>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>418.5</v>
+      </c>
+      <c r="I28" s="9" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>моносорт</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Эфиопия Иргач Гр.4 ТОП сухой /Эфиопи Милк (темн)</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>1815</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>1615</v>
+      </c>
+      <c r="G29" s="9" t="n">
+        <v>435</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>391.5</v>
+      </c>
+      <c r="I29" s="9" t="n">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>моносорт</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Эфиопия Лиму Гр.2 мытый</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>2120</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>1910</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>455</v>
+      </c>
+      <c r="H30" s="9" t="n">
+        <v>409.5</v>
+      </c>
+      <c r="I30" s="9" t="n">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>моносорт</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
           <t>Эфиопия Сидамо Гр.2 Гуджи мытый</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>E F</t>
         </is>
       </c>
-      <c r="D27" s="9" t="n">
+      <c r="D31" s="9" t="n">
         <v>2120</v>
       </c>
-      <c r="E27" s="9" t="n">
+      <c r="E31" s="9" t="n">
         <v>1910</v>
       </c>
-      <c r="F27" s="9" t="n">
+      <c r="F31" s="9" t="n">
         <v>1700</v>
       </c>
-      <c r="G27" s="9" t="n">
+      <c r="G31" s="9" t="n">
         <v>455</v>
       </c>
-      <c r="H27" s="9" t="n">
+      <c r="H31" s="9" t="n">
         <v>409.5</v>
       </c>
-      <c r="I27" s="9" t="n">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>🆕 моносорт</t>
-        </is>
-      </c>
-      <c r="B28" s="10" t="inlineStr">
-        <is>
-          <t>Китай Симао Гр.1 мытый</t>
-        </is>
-      </c>
-      <c r="C28" s="11" t="inlineStr">
-        <is>
-          <t>F E</t>
-        </is>
-      </c>
-      <c r="D28" s="12" t="n">
-        <v>2015</v>
-      </c>
-      <c r="E28" s="12" t="n">
-        <v>1815</v>
-      </c>
-      <c r="F28" s="12" t="n">
-        <v>1615</v>
-      </c>
-      <c r="G28" s="12" t="n">
-        <v>435</v>
-      </c>
-      <c r="H28" s="12" t="n">
-        <v>391.5</v>
-      </c>
-      <c r="I28" s="12" t="n">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>🆕 моносорт</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>Вьетнам Блю Шонла</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="inlineStr">
-        <is>
-          <t>F E</t>
-        </is>
-      </c>
-      <c r="D29" s="12" t="n">
-        <v>2135</v>
-      </c>
-      <c r="E29" s="12" t="n">
-        <v>1925</v>
-      </c>
-      <c r="F29" s="12" t="n">
-        <v>1710</v>
-      </c>
-      <c r="G29" s="12" t="n">
-        <v>455</v>
-      </c>
-      <c r="H29" s="12" t="n">
-        <v>409.5</v>
-      </c>
-      <c r="I29" s="12" t="n">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>🆕 моносорт</t>
-        </is>
-      </c>
-      <c r="B30" s="10" t="inlineStr">
-        <is>
-          <t>Коста-Рика Тарразу мытый</t>
-        </is>
-      </c>
-      <c r="C30" s="11" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D30" s="12" t="n">
-        <v>2250</v>
-      </c>
-      <c r="E30" s="12" t="n">
-        <v>2025</v>
-      </c>
-      <c r="F30" s="12" t="n">
-        <v>1800</v>
-      </c>
-      <c r="G30" s="12" t="n">
-        <v>480</v>
-      </c>
-      <c r="H30" s="12" t="n">
-        <v>432</v>
-      </c>
-      <c r="I30" s="12" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="10" t="inlineStr">
-        <is>
-          <t>🆕 моносорт</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>Гватемалла Грок</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>F E</t>
-        </is>
-      </c>
-      <c r="D31" s="12" t="n">
-        <v>2120</v>
-      </c>
-      <c r="E31" s="12" t="n">
-        <v>1910</v>
-      </c>
-      <c r="F31" s="12" t="n">
-        <v>1700</v>
-      </c>
-      <c r="G31" s="12" t="n">
-        <v>455</v>
-      </c>
-      <c r="H31" s="12" t="n">
-        <v>409.5</v>
-      </c>
-      <c r="I31" s="12" t="n">
+      <c r="I31" s="9" t="n">
         <v>364</v>
       </c>
     </row>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Эфиопия Челчеле гр.1 сухой</t>
+          <t>Эфиопия Иргач Челелекту мытый гр.1</t>
         </is>
       </c>
       <c r="C35" s="14" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>Эфиопия Иргач Челелекту мытый гр.1</t>
+          <t>Эфиопия Челчеле гр.1 сухой</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr">
@@ -1753,108 +1753,108 @@
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="13" t="inlineStr">
-        <is>
-          <t>микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>Колумбия Хайро Арсило сухой</t>
-        </is>
-      </c>
-      <c r="C37" s="14" t="inlineStr">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>🆕 микролот • BORЩ</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Бразилия SL28 Хани анаэроб.</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D37" s="15" t="n">
-        <v>2862.5</v>
-      </c>
-      <c r="E37" s="15" t="n">
-        <v>2580</v>
-      </c>
-      <c r="F37" s="15" t="n">
-        <v>2290</v>
-      </c>
-      <c r="G37" s="15" t="n">
-        <v>655</v>
-      </c>
-      <c r="H37" s="15" t="n">
-        <v>589.5</v>
-      </c>
-      <c r="I37" s="15" t="n">
-        <v>525</v>
+      <c r="D37" s="12" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E37" s="12" t="n">
+        <v>3150</v>
+      </c>
+      <c r="F37" s="12" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G37" s="12" t="n">
+        <v>780</v>
+      </c>
+      <c r="H37" s="12" t="n">
+        <v>702</v>
+      </c>
+      <c r="I37" s="12" t="n">
+        <v>625</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="13" t="inlineStr">
-        <is>
-          <t>микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>Колумбия Гонзало Кормана Катура сухой</t>
-        </is>
-      </c>
-      <c r="C38" s="14" t="inlineStr">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>🆕 микролот • BORЩ</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Бразилия Судан Руме анаэроб.</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D38" s="15" t="n">
+      <c r="D38" s="12" t="n">
         <v>3500</v>
       </c>
-      <c r="E38" s="15" t="n">
+      <c r="E38" s="12" t="n">
         <v>3150</v>
       </c>
-      <c r="F38" s="15" t="n">
+      <c r="F38" s="12" t="n">
         <v>2800</v>
       </c>
-      <c r="G38" s="15" t="n">
+      <c r="G38" s="12" t="n">
         <v>780</v>
       </c>
-      <c r="H38" s="15" t="n">
+      <c r="H38" s="12" t="n">
         <v>702</v>
       </c>
-      <c r="I38" s="15" t="n">
+      <c r="I38" s="12" t="n">
         <v>625</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="13" t="inlineStr">
-        <is>
-          <t>микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>Смесь Экваториальная</t>
-        </is>
-      </c>
-      <c r="C39" s="14" t="inlineStr">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>🆕 микролот • BORЩ</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Бразилия Фазенда Лагуинья мундо анаэроб.</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D39" s="15" t="n">
-        <v>3020</v>
-      </c>
-      <c r="E39" s="15" t="n">
-        <v>2720</v>
-      </c>
-      <c r="F39" s="15" t="n">
-        <v>2420</v>
-      </c>
-      <c r="G39" s="15" t="n">
-        <v>685</v>
-      </c>
-      <c r="H39" s="15" t="n">
-        <v>616.5</v>
-      </c>
-      <c r="I39" s="15" t="n">
-        <v>550</v>
+      <c r="D39" s="12" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E39" s="12" t="n">
+        <v>3150</v>
+      </c>
+      <c r="F39" s="12" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G39" s="12" t="n">
+        <v>780</v>
+      </c>
+      <c r="H39" s="12" t="n">
+        <v>702</v>
+      </c>
+      <c r="I39" s="12" t="n">
+        <v>625</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
@@ -1865,167 +1865,171 @@
       </c>
       <c r="B40" s="13" t="inlineStr">
         <is>
+          <t>Колумбия Гонзало Кормана Катура сухой</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E40" s="15" t="n">
+        <v>3150</v>
+      </c>
+      <c r="F40" s="15" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G40" s="15" t="n">
+        <v>780</v>
+      </c>
+      <c r="H40" s="15" t="n">
+        <v>702</v>
+      </c>
+      <c r="I40" s="15" t="n">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BORЩ</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>Колумбия Хайро Арсило сухой</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="n">
+        <v>2862.5</v>
+      </c>
+      <c r="E41" s="15" t="n">
+        <v>2580</v>
+      </c>
+      <c r="F41" s="15" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G41" s="15" t="n">
+        <v>655</v>
+      </c>
+      <c r="H41" s="15" t="n">
+        <v>589.5</v>
+      </c>
+      <c r="I41" s="15" t="n">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BORЩ</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>Смесь Экваториальная</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="n">
+        <v>3020</v>
+      </c>
+      <c r="E42" s="15" t="n">
+        <v>2720</v>
+      </c>
+      <c r="F42" s="15" t="n">
+        <v>2420</v>
+      </c>
+      <c r="G42" s="15" t="n">
+        <v>685</v>
+      </c>
+      <c r="H42" s="15" t="n">
+        <v>616.5</v>
+      </c>
+      <c r="I42" s="15" t="n">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BORЩ</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="inlineStr">
+        <is>
           <t>Эфиопия Арича гр.1 сухой</t>
         </is>
       </c>
-      <c r="C40" s="14" t="inlineStr">
+      <c r="C43" s="14" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D40" s="15" t="n">
+      <c r="D43" s="15" t="n">
         <v>3020</v>
       </c>
-      <c r="E40" s="15" t="n">
+      <c r="E43" s="15" t="n">
         <v>2720</v>
       </c>
-      <c r="F40" s="15" t="n">
+      <c r="F43" s="15" t="n">
         <v>2420</v>
       </c>
-      <c r="G40" s="15" t="n">
+      <c r="G43" s="15" t="n">
         <v>685</v>
       </c>
-      <c r="H40" s="15" t="n">
+      <c r="H43" s="15" t="n">
         <v>616.5</v>
       </c>
-      <c r="I40" s="15" t="n">
+      <c r="I43" s="15" t="n">
         <v>550</v>
       </c>
     </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>🆕 микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t>Бразилия SL28 Хани анаэроб.</t>
-        </is>
-      </c>
-      <c r="C41" s="11" t="inlineStr">
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>🆕 микролот</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>Колумбия Кастильо</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D41" s="12" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E41" s="12" t="n">
-        <v>3150</v>
-      </c>
-      <c r="F41" s="12" t="n">
-        <v>2800</v>
-      </c>
-      <c r="G41" s="12" t="n">
-        <v>780</v>
-      </c>
-      <c r="H41" s="12" t="n">
-        <v>702</v>
-      </c>
-      <c r="I41" s="12" t="n">
-        <v>625</v>
-      </c>
-    </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="10" t="inlineStr">
-        <is>
-          <t>🆕 микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B42" s="10" t="inlineStr">
-        <is>
-          <t>Бразилия Судан Руме анаэроб.</t>
-        </is>
-      </c>
-      <c r="C42" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D42" s="12" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E42" s="12" t="n">
-        <v>3150</v>
-      </c>
-      <c r="F42" s="12" t="n">
-        <v>2800</v>
-      </c>
-      <c r="G42" s="12" t="n">
-        <v>780</v>
-      </c>
-      <c r="H42" s="12" t="n">
-        <v>702</v>
-      </c>
-      <c r="I42" s="12" t="n">
-        <v>625</v>
-      </c>
-    </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="10" t="inlineStr">
-        <is>
-          <t>🆕 микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B43" s="10" t="inlineStr">
-        <is>
-          <t>Бразилия Фазенда Лагуинья мундо анаэроб.</t>
-        </is>
-      </c>
-      <c r="C43" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D43" s="12" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E43" s="12" t="n">
-        <v>3150</v>
-      </c>
-      <c r="F43" s="12" t="n">
-        <v>2800</v>
-      </c>
-      <c r="G43" s="12" t="n">
-        <v>780</v>
-      </c>
-      <c r="H43" s="12" t="n">
-        <v>702</v>
-      </c>
-      <c r="I43" s="12" t="n">
-        <v>625</v>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="13" t="inlineStr">
-        <is>
-          <t>микролот</t>
-        </is>
-      </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Колумбия Лили Роза Варгас Морено Чирозо Катуа </t>
-        </is>
-      </c>
-      <c r="C44" s="14" t="inlineStr"/>
-      <c r="D44" s="15" t="n">
-        <v>3102.5</v>
-      </c>
-      <c r="E44" s="15" t="n">
-        <v>2795</v>
-      </c>
-      <c r="F44" s="15" t="n">
-        <v>2485</v>
-      </c>
-      <c r="G44" s="15" t="n">
-        <v>700</v>
-      </c>
-      <c r="H44" s="15" t="n">
-        <v>630</v>
-      </c>
-      <c r="I44" s="15" t="n">
-        <v>560</v>
+      <c r="D44" s="12" t="n">
+        <v>2847.5</v>
+      </c>
+      <c r="E44" s="12" t="n">
+        <v>2565</v>
+      </c>
+      <c r="F44" s="12" t="n">
+        <v>2280</v>
+      </c>
+      <c r="G44" s="12" t="n">
+        <v>650</v>
+      </c>
+      <c r="H44" s="12" t="n">
+        <v>585</v>
+      </c>
+      <c r="I44" s="12" t="n">
+        <v>520</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
@@ -2036,194 +2040,190 @@
       </c>
       <c r="B45" s="13" t="inlineStr">
         <is>
-          <t>Колумбия Хиросос мытый</t>
+          <t xml:space="preserve">Колумбия Лили Роза Варгас Морено Чирозо Катуа </t>
         </is>
       </c>
       <c r="C45" s="14" t="inlineStr"/>
       <c r="D45" s="15" t="n">
+        <v>3102.5</v>
+      </c>
+      <c r="E45" s="15" t="n">
+        <v>2795</v>
+      </c>
+      <c r="F45" s="15" t="n">
+        <v>2485</v>
+      </c>
+      <c r="G45" s="15" t="n">
+        <v>700</v>
+      </c>
+      <c r="H45" s="15" t="n">
+        <v>630</v>
+      </c>
+      <c r="I45" s="15" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>🆕 микролот</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>Колумбия Маракуйя</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D46" s="12" t="n">
+        <v>5922.5</v>
+      </c>
+      <c r="E46" s="12" t="n">
+        <v>5335</v>
+      </c>
+      <c r="F46" s="12" t="n">
+        <v>4740</v>
+      </c>
+      <c r="G46" s="12" t="n">
+        <v>1265</v>
+      </c>
+      <c r="H46" s="12" t="n">
+        <v>1138.5</v>
+      </c>
+      <c r="I46" s="12" t="n">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>🆕 микролот</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>Колумбия Пачамама</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D47" s="12" t="n">
+        <v>4842.5</v>
+      </c>
+      <c r="E47" s="12" t="n">
+        <v>4360</v>
+      </c>
+      <c r="F47" s="12" t="n">
+        <v>3875</v>
+      </c>
+      <c r="G47" s="12" t="n">
+        <v>1050</v>
+      </c>
+      <c r="H47" s="12" t="n">
+        <v>945</v>
+      </c>
+      <c r="I47" s="12" t="n">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>микролот</t>
+        </is>
+      </c>
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>Колумбия Хиросос мытый</t>
+        </is>
+      </c>
+      <c r="C48" s="14" t="inlineStr"/>
+      <c r="D48" s="15" t="n">
         <v>2547.5</v>
       </c>
-      <c r="E45" s="15" t="n">
+      <c r="E48" s="15" t="n">
         <v>2295</v>
       </c>
-      <c r="F45" s="15" t="n">
+      <c r="F48" s="15" t="n">
         <v>2040</v>
       </c>
-      <c r="G45" s="15" t="n">
+      <c r="G48" s="15" t="n">
         <v>590</v>
       </c>
-      <c r="H45" s="15" t="n">
+      <c r="H48" s="15" t="n">
         <v>531</v>
       </c>
-      <c r="I45" s="15" t="n">
+      <c r="I48" s="15" t="n">
         <v>475</v>
       </c>
     </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="13" t="inlineStr">
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="13" t="inlineStr">
         <is>
           <t>микролот</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>КолумбияХайро Асрило инфьюз Маракуйя</t>
+        </is>
+      </c>
+      <c r="C49" s="14" t="inlineStr"/>
+      <c r="D49" s="15" t="n">
+        <v>4925</v>
+      </c>
+      <c r="E49" s="15" t="n">
+        <v>4435</v>
+      </c>
+      <c r="F49" s="15" t="n">
+        <v>3940</v>
+      </c>
+      <c r="G49" s="15" t="n">
+        <v>1065</v>
+      </c>
+      <c r="H49" s="15" t="n">
+        <v>958.5</v>
+      </c>
+      <c r="I49" s="15" t="n">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>микролот</t>
+        </is>
+      </c>
+      <c r="B50" s="13" t="inlineStr">
         <is>
           <t>Руанада Нямашеки хилс сухой</t>
         </is>
       </c>
-      <c r="C46" s="14" t="inlineStr"/>
-      <c r="D46" s="15" t="n">
+      <c r="C50" s="14" t="inlineStr"/>
+      <c r="D50" s="15" t="n">
         <v>2862.5</v>
       </c>
-      <c r="E46" s="15" t="n">
+      <c r="E50" s="15" t="n">
         <v>2580</v>
       </c>
-      <c r="F46" s="15" t="n">
+      <c r="F50" s="15" t="n">
         <v>2290</v>
       </c>
-      <c r="G46" s="15" t="n">
+      <c r="G50" s="15" t="n">
         <v>655</v>
       </c>
-      <c r="H46" s="15" t="n">
+      <c r="H50" s="15" t="n">
         <v>589.5</v>
       </c>
-      <c r="I46" s="15" t="n">
+      <c r="I50" s="15" t="n">
         <v>525</v>
-      </c>
-    </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="13" t="inlineStr">
-        <is>
-          <t>микролот</t>
-        </is>
-      </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>КолумбияХайро Асрило инфьюз Маракуйя</t>
-        </is>
-      </c>
-      <c r="C47" s="14" t="inlineStr"/>
-      <c r="D47" s="15" t="n">
-        <v>4925</v>
-      </c>
-      <c r="E47" s="15" t="n">
-        <v>4435</v>
-      </c>
-      <c r="F47" s="15" t="n">
-        <v>3940</v>
-      </c>
-      <c r="G47" s="15" t="n">
-        <v>1065</v>
-      </c>
-      <c r="H47" s="15" t="n">
-        <v>958.5</v>
-      </c>
-      <c r="I47" s="15" t="n">
-        <v>855</v>
-      </c>
-    </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="10" t="inlineStr">
-        <is>
-          <t>🆕 микролот</t>
-        </is>
-      </c>
-      <c r="B48" s="10" t="inlineStr">
-        <is>
-          <t>Колумбия Кастильо</t>
-        </is>
-      </c>
-      <c r="C48" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D48" s="12" t="n">
-        <v>2847.5</v>
-      </c>
-      <c r="E48" s="12" t="n">
-        <v>2565</v>
-      </c>
-      <c r="F48" s="12" t="n">
-        <v>2280</v>
-      </c>
-      <c r="G48" s="12" t="n">
-        <v>650</v>
-      </c>
-      <c r="H48" s="12" t="n">
-        <v>585</v>
-      </c>
-      <c r="I48" s="12" t="n">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="10" t="inlineStr">
-        <is>
-          <t>🆕 микролот</t>
-        </is>
-      </c>
-      <c r="B49" s="10" t="inlineStr">
-        <is>
-          <t>Колумбия Пачамама</t>
-        </is>
-      </c>
-      <c r="C49" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D49" s="12" t="n">
-        <v>4842.5</v>
-      </c>
-      <c r="E49" s="12" t="n">
-        <v>4360</v>
-      </c>
-      <c r="F49" s="12" t="n">
-        <v>3875</v>
-      </c>
-      <c r="G49" s="12" t="n">
-        <v>1050</v>
-      </c>
-      <c r="H49" s="12" t="n">
-        <v>945</v>
-      </c>
-      <c r="I49" s="12" t="n">
-        <v>840</v>
-      </c>
-    </row>
-    <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="10" t="inlineStr">
-        <is>
-          <t>🆕 микролот</t>
-        </is>
-      </c>
-      <c r="B50" s="10" t="inlineStr">
-        <is>
-          <t>Колумбия Маракуйя</t>
-        </is>
-      </c>
-      <c r="C50" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D50" s="12" t="n">
-        <v>5922.5</v>
-      </c>
-      <c r="E50" s="12" t="n">
-        <v>5335</v>
-      </c>
-      <c r="F50" s="12" t="n">
-        <v>4740</v>
-      </c>
-      <c r="G50" s="12" t="n">
-        <v>1265</v>
-      </c>
-      <c r="H50" s="12" t="n">
-        <v>1138.5</v>
-      </c>
-      <c r="I50" s="12" t="n">
-        <v>1015</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bishop: Auto stock sync from 1C: stock updates 12
</commit_message>
<xml_diff>
--- a/tma_static/data/Roastberry_Прайс_2026.xlsx
+++ b/tma_static/data/Roastberry_Прайс_2026.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прайс 2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Прайс 2026" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -79,12 +79,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -143,22 +143,22 @@
     <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -614,22 +614,22 @@
       </c>
       <c r="C4" s="5" t="inlineStr"/>
       <c r="D4" s="6" t="n">
-        <v>1975</v>
+        <v>1875</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>1780</v>
+        <v>1690</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>1580</v>
+        <v>1500</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>425</v>
+        <v>405</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>382.5</v>
+        <v>364.5</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>340</v>
+        <v>324</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -649,22 +649,22 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>1910</v>
+        <v>1815</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>1720</v>
+        <v>1635</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>1530</v>
+        <v>1455</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>410</v>
+        <v>395</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>369</v>
+        <v>355.5</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>328</v>
+        <v>316</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
@@ -684,22 +684,22 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>2015</v>
+        <v>1910</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>1815</v>
+        <v>1720</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>1615</v>
+        <v>1530</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>435</v>
+        <v>410</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>391.5</v>
+        <v>369</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>348</v>
+        <v>328</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
@@ -719,22 +719,22 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>2015</v>
+        <v>1910</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>1815</v>
+        <v>1720</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>1615</v>
+        <v>1530</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>435</v>
+        <v>410</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>391.5</v>
+        <v>369</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>348</v>
+        <v>328</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -754,22 +754,22 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>2015</v>
+        <v>1910</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>1815</v>
+        <v>1720</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>1615</v>
+        <v>1530</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>435</v>
+        <v>410</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>391.5</v>
+        <v>369</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>348</v>
+        <v>328</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -789,22 +789,22 @@
         </is>
       </c>
       <c r="D9" s="9" t="n">
-        <v>2070</v>
+        <v>1960</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>1865</v>
+        <v>1765</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>1660</v>
+        <v>1570</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>445</v>
+        <v>420</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>400.5</v>
+        <v>378</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>356</v>
+        <v>336</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -824,22 +824,22 @@
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>2120</v>
+        <v>2005</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>1910</v>
+        <v>1805</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>1700</v>
+        <v>1605</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>455</v>
+        <v>430</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>409.5</v>
+        <v>387</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>364</v>
+        <v>344</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
@@ -859,92 +859,92 @@
         </is>
       </c>
       <c r="D11" s="9" t="n">
+        <v>1910</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>1720</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>1530</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>410</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>369</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>моносорт</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Вьетнам Блю Шонла</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>F E</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="n">
         <v>2015</v>
       </c>
-      <c r="E11" s="9" t="n">
+      <c r="E12" s="9" t="n">
         <v>1815</v>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F12" s="9" t="n">
         <v>1615</v>
       </c>
-      <c r="G11" s="9" t="n">
+      <c r="G12" s="9" t="n">
         <v>435</v>
       </c>
-      <c r="H11" s="9" t="n">
+      <c r="H12" s="9" t="n">
         <v>391.5</v>
       </c>
-      <c r="I11" s="9" t="n">
+      <c r="I12" s="9" t="n">
         <v>348</v>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>🆕 моносорт</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Вьетнам Блю Шонла</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>моносорт</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Гватемалла Грок</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>F E</t>
         </is>
       </c>
-      <c r="D12" s="12" t="n">
-        <v>2135</v>
-      </c>
-      <c r="E12" s="12" t="n">
-        <v>1925</v>
-      </c>
-      <c r="F12" s="12" t="n">
-        <v>1710</v>
-      </c>
-      <c r="G12" s="12" t="n">
-        <v>455</v>
-      </c>
-      <c r="H12" s="12" t="n">
-        <v>409.5</v>
-      </c>
-      <c r="I12" s="12" t="n">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>🆕 моносорт</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Гватемалла Грок</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>F E</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="n">
-        <v>2120</v>
-      </c>
-      <c r="E13" s="12" t="n">
-        <v>1910</v>
-      </c>
-      <c r="F13" s="12" t="n">
-        <v>1700</v>
-      </c>
-      <c r="G13" s="12" t="n">
-        <v>455</v>
-      </c>
-      <c r="H13" s="12" t="n">
-        <v>409.5</v>
-      </c>
-      <c r="I13" s="12" t="n">
-        <v>364</v>
+      <c r="D13" s="9" t="n">
+        <v>2005</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>1805</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>1605</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>430</v>
+      </c>
+      <c r="H13" s="9" t="n">
+        <v>387</v>
+      </c>
+      <c r="I13" s="9" t="n">
+        <v>344</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
@@ -964,22 +964,22 @@
         </is>
       </c>
       <c r="D14" s="9" t="n">
-        <v>2440</v>
+        <v>2295</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>2200</v>
+        <v>2070</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>1955</v>
+        <v>1840</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>520</v>
+        <v>490</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>468</v>
+        <v>441</v>
       </c>
       <c r="I14" s="9" t="n">
-        <v>416</v>
+        <v>392</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -999,22 +999,22 @@
         </is>
       </c>
       <c r="D15" s="9" t="n">
-        <v>2175</v>
+        <v>2055</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>1960</v>
+        <v>1850</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>1740</v>
+        <v>1645</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>465</v>
+        <v>440</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>418.5</v>
+        <v>396</v>
       </c>
       <c r="I15" s="9" t="n">
-        <v>372</v>
+        <v>352</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
@@ -1034,22 +1034,22 @@
         </is>
       </c>
       <c r="D16" s="9" t="n">
-        <v>2595</v>
+        <v>2440</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>2340</v>
+        <v>2200</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>2080</v>
+        <v>1955</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>550</v>
+        <v>520</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>495</v>
+        <v>468</v>
       </c>
       <c r="I16" s="9" t="n">
-        <v>440</v>
+        <v>416</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
@@ -1069,22 +1069,22 @@
         </is>
       </c>
       <c r="D17" s="9" t="n">
-        <v>2490</v>
+        <v>2345</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>2245</v>
+        <v>2115</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>1995</v>
+        <v>1880</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>530</v>
+        <v>500</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>477</v>
+        <v>450</v>
       </c>
       <c r="I17" s="9" t="n">
-        <v>424</v>
+        <v>400</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
@@ -1104,22 +1104,22 @@
         </is>
       </c>
       <c r="D18" s="9" t="n">
-        <v>2015</v>
+        <v>1910</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>1815</v>
+        <v>1720</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>1615</v>
+        <v>1530</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>435</v>
+        <v>410</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>391.5</v>
+        <v>369</v>
       </c>
       <c r="I18" s="9" t="n">
-        <v>348</v>
+        <v>328</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
@@ -1139,57 +1139,57 @@
         </is>
       </c>
       <c r="D19" s="9" t="n">
-        <v>2175</v>
+        <v>2055</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>1960</v>
+        <v>1850</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>1740</v>
+        <v>1645</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>465</v>
+        <v>440</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>418.5</v>
+        <v>396</v>
       </c>
       <c r="I19" s="9" t="n">
-        <v>372</v>
+        <v>352</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>🆕 моносорт</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>моносорт</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Коста-Рика Тарразу мытый</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D20" s="12" t="n">
-        <v>2250</v>
-      </c>
-      <c r="E20" s="12" t="n">
-        <v>2025</v>
-      </c>
-      <c r="F20" s="12" t="n">
-        <v>1800</v>
-      </c>
-      <c r="G20" s="12" t="n">
-        <v>480</v>
-      </c>
-      <c r="H20" s="12" t="n">
-        <v>432</v>
-      </c>
-      <c r="I20" s="12" t="n">
-        <v>384</v>
+      <c r="D20" s="9" t="n">
+        <v>2120</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>1910</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>455</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>409.5</v>
+      </c>
+      <c r="I20" s="9" t="n">
+        <v>364</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
@@ -1209,22 +1209,22 @@
         </is>
       </c>
       <c r="D21" s="9" t="n">
-        <v>2545</v>
+        <v>2390</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>2295</v>
+        <v>2155</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>2040</v>
+        <v>1915</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>540</v>
+        <v>510</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>486</v>
+        <v>459</v>
       </c>
       <c r="I21" s="9" t="n">
-        <v>432</v>
+        <v>408</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
@@ -1244,22 +1244,22 @@
         </is>
       </c>
       <c r="D22" s="9" t="n">
-        <v>2230</v>
+        <v>2105</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>2010</v>
+        <v>1895</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>1785</v>
+        <v>1685</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>475</v>
+        <v>450</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>427.5</v>
+        <v>405</v>
       </c>
       <c r="I22" s="9" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
@@ -1279,22 +1279,22 @@
         </is>
       </c>
       <c r="D23" s="9" t="n">
-        <v>2620</v>
+        <v>2460</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>2360</v>
+        <v>2215</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>2100</v>
+        <v>1970</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>555</v>
+        <v>520</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>499.5</v>
+        <v>468</v>
       </c>
       <c r="I23" s="9" t="n">
-        <v>444</v>
+        <v>416</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
@@ -1314,22 +1314,22 @@
         </is>
       </c>
       <c r="D24" s="9" t="n">
-        <v>2230</v>
+        <v>2105</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>2010</v>
+        <v>1895</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>1785</v>
+        <v>1685</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>475</v>
+        <v>450</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>427.5</v>
+        <v>405</v>
       </c>
       <c r="I24" s="9" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
@@ -1349,22 +1349,22 @@
         </is>
       </c>
       <c r="D25" s="9" t="n">
-        <v>2335</v>
+        <v>2200</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>2105</v>
+        <v>1980</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>1870</v>
+        <v>1760</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>495</v>
+        <v>470</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>445.5</v>
+        <v>423</v>
       </c>
       <c r="I25" s="9" t="n">
-        <v>396</v>
+        <v>376</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
@@ -1384,22 +1384,22 @@
         </is>
       </c>
       <c r="D26" s="9" t="n">
-        <v>2070</v>
+        <v>1960</v>
       </c>
       <c r="E26" s="9" t="n">
-        <v>1865</v>
+        <v>1765</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>1660</v>
+        <v>1570</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>445</v>
+        <v>420</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>400.5</v>
+        <v>378</v>
       </c>
       <c r="I26" s="9" t="n">
-        <v>356</v>
+        <v>336</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
@@ -1419,22 +1419,22 @@
         </is>
       </c>
       <c r="D27" s="9" t="n">
-        <v>2015</v>
+        <v>1910</v>
       </c>
       <c r="E27" s="9" t="n">
-        <v>1815</v>
+        <v>1720</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>1615</v>
+        <v>1530</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>435</v>
+        <v>410</v>
       </c>
       <c r="H27" s="9" t="n">
-        <v>391.5</v>
+        <v>369</v>
       </c>
       <c r="I27" s="9" t="n">
-        <v>348</v>
+        <v>328</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
@@ -1454,22 +1454,22 @@
         </is>
       </c>
       <c r="D28" s="9" t="n">
-        <v>2175</v>
+        <v>2055</v>
       </c>
       <c r="E28" s="9" t="n">
-        <v>1960</v>
+        <v>1850</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>1740</v>
+        <v>1645</v>
       </c>
       <c r="G28" s="9" t="n">
-        <v>465</v>
+        <v>440</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>418.5</v>
+        <v>396</v>
       </c>
       <c r="I28" s="9" t="n">
-        <v>372</v>
+        <v>352</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
@@ -1489,22 +1489,22 @@
         </is>
       </c>
       <c r="D29" s="9" t="n">
-        <v>2015</v>
+        <v>1910</v>
       </c>
       <c r="E29" s="9" t="n">
-        <v>1815</v>
+        <v>1720</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>1615</v>
+        <v>1530</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>435</v>
+        <v>410</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>391.5</v>
+        <v>369</v>
       </c>
       <c r="I29" s="9" t="n">
-        <v>348</v>
+        <v>328</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
@@ -1524,22 +1524,22 @@
         </is>
       </c>
       <c r="D30" s="9" t="n">
-        <v>2120</v>
+        <v>2005</v>
       </c>
       <c r="E30" s="9" t="n">
-        <v>1910</v>
+        <v>1805</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>1700</v>
+        <v>1605</v>
       </c>
       <c r="G30" s="9" t="n">
-        <v>455</v>
+        <v>430</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>409.5</v>
+        <v>387</v>
       </c>
       <c r="I30" s="9" t="n">
-        <v>364</v>
+        <v>344</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
@@ -1559,518 +1559,518 @@
         </is>
       </c>
       <c r="D31" s="9" t="n">
-        <v>2120</v>
+        <v>2005</v>
       </c>
       <c r="E31" s="9" t="n">
-        <v>1910</v>
+        <v>1805</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>1700</v>
+        <v>1605</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>455</v>
+        <v>430</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>409.5</v>
+        <v>387</v>
       </c>
       <c r="I31" s="9" t="n">
-        <v>364</v>
+        <v>344</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="13" t="inlineStr">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B32" s="13" t="inlineStr">
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>Колумбия Клаудиа Колменарес Гейша мытый</t>
         </is>
       </c>
-      <c r="C32" s="14" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D32" s="15" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E32" s="15" t="n">
-        <v>3150</v>
-      </c>
-      <c r="F32" s="15" t="n">
-        <v>2800</v>
-      </c>
-      <c r="G32" s="15" t="n">
-        <v>780</v>
-      </c>
-      <c r="H32" s="15" t="n">
-        <v>702</v>
-      </c>
-      <c r="I32" s="15" t="n">
-        <v>625</v>
+      <c r="D32" s="12" t="n">
+        <v>3192.5</v>
+      </c>
+      <c r="E32" s="12" t="n">
+        <v>2875</v>
+      </c>
+      <c r="F32" s="12" t="n">
+        <v>2555</v>
+      </c>
+      <c r="G32" s="12" t="n">
+        <v>720</v>
+      </c>
+      <c r="H32" s="12" t="n">
+        <v>648</v>
+      </c>
+      <c r="I32" s="12" t="n">
+        <v>580</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="A33" s="10" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>Эфиопия Иргач Адада гр.1 сухой</t>
         </is>
       </c>
-      <c r="C33" s="14" t="inlineStr">
+      <c r="C33" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D33" s="15" t="n">
-        <v>2390</v>
-      </c>
-      <c r="E33" s="15" t="n">
-        <v>2155</v>
-      </c>
-      <c r="F33" s="15" t="n">
-        <v>1915</v>
-      </c>
-      <c r="G33" s="15" t="n">
-        <v>560</v>
-      </c>
-      <c r="H33" s="15" t="n">
-        <v>504</v>
-      </c>
-      <c r="I33" s="15" t="n">
-        <v>450</v>
+      <c r="D33" s="12" t="n">
+        <v>2187.5</v>
+      </c>
+      <c r="E33" s="12" t="n">
+        <v>1970</v>
+      </c>
+      <c r="F33" s="12" t="n">
+        <v>1750</v>
+      </c>
+      <c r="G33" s="12" t="n">
+        <v>520</v>
+      </c>
+      <c r="H33" s="12" t="n">
+        <v>468</v>
+      </c>
+      <c r="I33" s="12" t="n">
+        <v>420</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="A34" s="10" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>Эфиопия Иргач Билоя гр.2 сухой</t>
         </is>
       </c>
-      <c r="C34" s="14" t="inlineStr">
+      <c r="C34" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D34" s="15" t="n">
-        <v>2232.5</v>
-      </c>
-      <c r="E34" s="15" t="n">
-        <v>2010</v>
-      </c>
-      <c r="F34" s="15" t="n">
-        <v>1790</v>
-      </c>
-      <c r="G34" s="15" t="n">
-        <v>525</v>
-      </c>
-      <c r="H34" s="15" t="n">
-        <v>472.5</v>
-      </c>
-      <c r="I34" s="15" t="n">
-        <v>420</v>
+      <c r="D34" s="12" t="n">
+        <v>2045</v>
+      </c>
+      <c r="E34" s="12" t="n">
+        <v>1845</v>
+      </c>
+      <c r="F34" s="12" t="n">
+        <v>1640</v>
+      </c>
+      <c r="G34" s="12" t="n">
+        <v>490</v>
+      </c>
+      <c r="H34" s="12" t="n">
+        <v>441</v>
+      </c>
+      <c r="I34" s="12" t="n">
+        <v>395</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="13" t="inlineStr">
+      <c r="A35" s="10" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="10" t="inlineStr">
         <is>
           <t>Эфиопия Иргач Челелекту мытый гр.1</t>
         </is>
       </c>
-      <c r="C35" s="14" t="inlineStr">
+      <c r="C35" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D35" s="15" t="n">
-        <v>2862.5</v>
-      </c>
-      <c r="E35" s="15" t="n">
-        <v>2580</v>
-      </c>
-      <c r="F35" s="15" t="n">
-        <v>2290</v>
-      </c>
-      <c r="G35" s="15" t="n">
-        <v>655</v>
-      </c>
-      <c r="H35" s="15" t="n">
-        <v>589.5</v>
-      </c>
-      <c r="I35" s="15" t="n">
-        <v>525</v>
+      <c r="D35" s="12" t="n">
+        <v>2615</v>
+      </c>
+      <c r="E35" s="12" t="n">
+        <v>2355</v>
+      </c>
+      <c r="F35" s="12" t="n">
+        <v>2095</v>
+      </c>
+      <c r="G35" s="12" t="n">
+        <v>605</v>
+      </c>
+      <c r="H35" s="12" t="n">
+        <v>544.5</v>
+      </c>
+      <c r="I35" s="12" t="n">
+        <v>485</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="13" t="inlineStr">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>Эфиопия Челчеле гр.1 сухой</t>
         </is>
       </c>
-      <c r="C36" s="14" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D36" s="15" t="n">
-        <v>2862.5</v>
-      </c>
-      <c r="E36" s="15" t="n">
-        <v>2580</v>
-      </c>
-      <c r="F36" s="15" t="n">
-        <v>2290</v>
-      </c>
-      <c r="G36" s="15" t="n">
-        <v>655</v>
-      </c>
-      <c r="H36" s="15" t="n">
-        <v>589.5</v>
-      </c>
-      <c r="I36" s="15" t="n">
-        <v>525</v>
+      <c r="D36" s="12" t="n">
+        <v>2615</v>
+      </c>
+      <c r="E36" s="12" t="n">
+        <v>2355</v>
+      </c>
+      <c r="F36" s="12" t="n">
+        <v>2095</v>
+      </c>
+      <c r="G36" s="12" t="n">
+        <v>605</v>
+      </c>
+      <c r="H36" s="12" t="n">
+        <v>544.5</v>
+      </c>
+      <c r="I36" s="12" t="n">
+        <v>485</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="A37" s="10" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
+      <c r="B37" s="10" t="inlineStr">
         <is>
           <t>Бразилия SL28 Хани анаэроб.</t>
         </is>
       </c>
-      <c r="C37" s="14" t="inlineStr">
+      <c r="C37" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D37" s="15" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E37" s="15" t="n">
-        <v>3150</v>
-      </c>
-      <c r="F37" s="15" t="n">
-        <v>2800</v>
-      </c>
-      <c r="G37" s="15" t="n">
-        <v>780</v>
-      </c>
-      <c r="H37" s="15" t="n">
-        <v>702</v>
-      </c>
-      <c r="I37" s="15" t="n">
-        <v>625</v>
+      <c r="D37" s="12" t="n">
+        <v>3192.5</v>
+      </c>
+      <c r="E37" s="12" t="n">
+        <v>2875</v>
+      </c>
+      <c r="F37" s="12" t="n">
+        <v>2555</v>
+      </c>
+      <c r="G37" s="12" t="n">
+        <v>720</v>
+      </c>
+      <c r="H37" s="12" t="n">
+        <v>648</v>
+      </c>
+      <c r="I37" s="12" t="n">
+        <v>580</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="A38" s="10" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
+      <c r="B38" s="10" t="inlineStr">
         <is>
           <t>Бразилия Судан Руме анаэроб.</t>
         </is>
       </c>
-      <c r="C38" s="14" t="inlineStr">
+      <c r="C38" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D38" s="15" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E38" s="15" t="n">
-        <v>3150</v>
-      </c>
-      <c r="F38" s="15" t="n">
-        <v>2800</v>
-      </c>
-      <c r="G38" s="15" t="n">
-        <v>780</v>
-      </c>
-      <c r="H38" s="15" t="n">
-        <v>702</v>
-      </c>
-      <c r="I38" s="15" t="n">
-        <v>625</v>
+      <c r="D38" s="12" t="n">
+        <v>3192.5</v>
+      </c>
+      <c r="E38" s="12" t="n">
+        <v>2875</v>
+      </c>
+      <c r="F38" s="12" t="n">
+        <v>2555</v>
+      </c>
+      <c r="G38" s="12" t="n">
+        <v>720</v>
+      </c>
+      <c r="H38" s="12" t="n">
+        <v>648</v>
+      </c>
+      <c r="I38" s="12" t="n">
+        <v>580</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="A39" s="10" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
+      <c r="B39" s="10" t="inlineStr">
         <is>
           <t>Бразилия Фазенда Лагуинья мундо анаэроб.</t>
         </is>
       </c>
-      <c r="C39" s="14" t="inlineStr">
+      <c r="C39" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D39" s="15" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E39" s="15" t="n">
-        <v>3150</v>
-      </c>
-      <c r="F39" s="15" t="n">
-        <v>2800</v>
-      </c>
-      <c r="G39" s="15" t="n">
-        <v>780</v>
-      </c>
-      <c r="H39" s="15" t="n">
-        <v>702</v>
-      </c>
-      <c r="I39" s="15" t="n">
-        <v>625</v>
+      <c r="D39" s="12" t="n">
+        <v>3192.5</v>
+      </c>
+      <c r="E39" s="12" t="n">
+        <v>2875</v>
+      </c>
+      <c r="F39" s="12" t="n">
+        <v>2555</v>
+      </c>
+      <c r="G39" s="12" t="n">
+        <v>720</v>
+      </c>
+      <c r="H39" s="12" t="n">
+        <v>648</v>
+      </c>
+      <c r="I39" s="12" t="n">
+        <v>580</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="13" t="inlineStr">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
+      <c r="B40" s="10" t="inlineStr">
         <is>
           <t>Колумбия Гонзало Кормана Катура сухой</t>
         </is>
       </c>
-      <c r="C40" s="14" t="inlineStr">
+      <c r="C40" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D40" s="15" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E40" s="15" t="n">
-        <v>3150</v>
-      </c>
-      <c r="F40" s="15" t="n">
-        <v>2800</v>
-      </c>
-      <c r="G40" s="15" t="n">
-        <v>780</v>
-      </c>
-      <c r="H40" s="15" t="n">
-        <v>702</v>
-      </c>
-      <c r="I40" s="15" t="n">
-        <v>625</v>
+      <c r="D40" s="12" t="n">
+        <v>3192.5</v>
+      </c>
+      <c r="E40" s="12" t="n">
+        <v>2875</v>
+      </c>
+      <c r="F40" s="12" t="n">
+        <v>2555</v>
+      </c>
+      <c r="G40" s="12" t="n">
+        <v>720</v>
+      </c>
+      <c r="H40" s="12" t="n">
+        <v>648</v>
+      </c>
+      <c r="I40" s="12" t="n">
+        <v>580</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="13" t="inlineStr">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
+      <c r="B41" s="10" t="inlineStr">
         <is>
           <t>Колумбия Хайро Арсило сухой</t>
         </is>
       </c>
-      <c r="C41" s="14" t="inlineStr">
+      <c r="C41" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D41" s="15" t="n">
-        <v>2862.5</v>
-      </c>
-      <c r="E41" s="15" t="n">
-        <v>2580</v>
-      </c>
-      <c r="F41" s="15" t="n">
-        <v>2290</v>
-      </c>
-      <c r="G41" s="15" t="n">
-        <v>655</v>
-      </c>
-      <c r="H41" s="15" t="n">
-        <v>589.5</v>
-      </c>
-      <c r="I41" s="15" t="n">
-        <v>525</v>
+      <c r="D41" s="12" t="n">
+        <v>2615</v>
+      </c>
+      <c r="E41" s="12" t="n">
+        <v>2355</v>
+      </c>
+      <c r="F41" s="12" t="n">
+        <v>2095</v>
+      </c>
+      <c r="G41" s="12" t="n">
+        <v>605</v>
+      </c>
+      <c r="H41" s="12" t="n">
+        <v>544.5</v>
+      </c>
+      <c r="I41" s="12" t="n">
+        <v>485</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="13" t="inlineStr">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
+      <c r="B42" s="10" t="inlineStr">
         <is>
           <t>Смесь Экваториальная</t>
         </is>
       </c>
-      <c r="C42" s="14" t="inlineStr">
+      <c r="C42" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D42" s="15" t="n">
-        <v>3020</v>
-      </c>
-      <c r="E42" s="15" t="n">
-        <v>2720</v>
-      </c>
-      <c r="F42" s="15" t="n">
-        <v>2420</v>
-      </c>
-      <c r="G42" s="15" t="n">
-        <v>685</v>
-      </c>
-      <c r="H42" s="15" t="n">
-        <v>616.5</v>
-      </c>
-      <c r="I42" s="15" t="n">
-        <v>550</v>
+      <c r="D42" s="12" t="n">
+        <v>2765</v>
+      </c>
+      <c r="E42" s="12" t="n">
+        <v>2490</v>
+      </c>
+      <c r="F42" s="12" t="n">
+        <v>2215</v>
+      </c>
+      <c r="G42" s="12" t="n">
+        <v>635</v>
+      </c>
+      <c r="H42" s="12" t="n">
+        <v>571.5</v>
+      </c>
+      <c r="I42" s="12" t="n">
+        <v>510</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="13" t="inlineStr">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
+      <c r="B43" s="10" t="inlineStr">
         <is>
           <t>Эфиопия Арича гр.1 сухой</t>
         </is>
       </c>
-      <c r="C43" s="14" t="inlineStr">
+      <c r="C43" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D43" s="15" t="n">
-        <v>3020</v>
-      </c>
-      <c r="E43" s="15" t="n">
-        <v>2720</v>
-      </c>
-      <c r="F43" s="15" t="n">
-        <v>2420</v>
-      </c>
-      <c r="G43" s="15" t="n">
-        <v>685</v>
-      </c>
-      <c r="H43" s="15" t="n">
-        <v>616.5</v>
-      </c>
-      <c r="I43" s="15" t="n">
-        <v>550</v>
+      <c r="D43" s="12" t="n">
+        <v>2765</v>
+      </c>
+      <c r="E43" s="12" t="n">
+        <v>2490</v>
+      </c>
+      <c r="F43" s="12" t="n">
+        <v>2215</v>
+      </c>
+      <c r="G43" s="12" t="n">
+        <v>635</v>
+      </c>
+      <c r="H43" s="12" t="n">
+        <v>571.5</v>
+      </c>
+      <c r="I43" s="12" t="n">
+        <v>510</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="10" t="inlineStr">
+      <c r="A44" s="13" t="inlineStr">
         <is>
           <t>🆕 микролот</t>
         </is>
       </c>
-      <c r="B44" s="10" t="inlineStr">
+      <c r="B44" s="13" t="inlineStr">
         <is>
           <t>Кения КиаваМуруру нат.анаэроб.</t>
         </is>
       </c>
-      <c r="C44" s="11" t="inlineStr">
+      <c r="C44" s="14" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D44" s="12" t="n">
-        <v>3972.5</v>
-      </c>
-      <c r="E44" s="12" t="n">
-        <v>3580</v>
-      </c>
-      <c r="F44" s="12" t="n">
-        <v>3180</v>
-      </c>
-      <c r="G44" s="12" t="n">
-        <v>875</v>
-      </c>
-      <c r="H44" s="12" t="n">
-        <v>787.5</v>
-      </c>
-      <c r="I44" s="12" t="n">
-        <v>700</v>
+      <c r="D44" s="15" t="n">
+        <v>3627.5</v>
+      </c>
+      <c r="E44" s="15" t="n">
+        <v>3265</v>
+      </c>
+      <c r="F44" s="15" t="n">
+        <v>2905</v>
+      </c>
+      <c r="G44" s="15" t="n">
+        <v>805</v>
+      </c>
+      <c r="H44" s="15" t="n">
+        <v>724.5</v>
+      </c>
+      <c r="I44" s="15" t="n">
+        <v>645</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="10" t="inlineStr">
+      <c r="A45" s="13" t="inlineStr">
         <is>
           <t>🆕 микролот</t>
         </is>
       </c>
-      <c r="B45" s="10" t="inlineStr">
+      <c r="B45" s="13" t="inlineStr">
         <is>
           <t>Кения Маакиоу Пиберри</t>
         </is>
       </c>
-      <c r="C45" s="11" t="inlineStr">
+      <c r="C45" s="14" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D45" s="12" t="n">
-        <v>2960</v>
-      </c>
-      <c r="E45" s="12" t="n">
-        <v>2665</v>
-      </c>
-      <c r="F45" s="12" t="n">
-        <v>2370</v>
-      </c>
-      <c r="G45" s="12" t="n">
-        <v>670</v>
-      </c>
-      <c r="H45" s="12" t="n">
-        <v>603</v>
-      </c>
-      <c r="I45" s="12" t="n">
-        <v>540</v>
+      <c r="D45" s="15" t="n">
+        <v>2705</v>
+      </c>
+      <c r="E45" s="15" t="n">
+        <v>2435</v>
+      </c>
+      <c r="F45" s="15" t="n">
+        <v>2165</v>
+      </c>
+      <c r="G45" s="15" t="n">
+        <v>620</v>
+      </c>
+      <c r="H45" s="15" t="n">
+        <v>558</v>
+      </c>
+      <c r="I45" s="15" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>🆕 микролот</t>
+          <t>микролот</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
@@ -2084,59 +2084,59 @@
         </is>
       </c>
       <c r="D46" s="12" t="n">
-        <v>2847.5</v>
+        <v>2600</v>
       </c>
       <c r="E46" s="12" t="n">
-        <v>2565</v>
+        <v>2340</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>2280</v>
+        <v>2080</v>
       </c>
       <c r="G46" s="12" t="n">
-        <v>650</v>
+        <v>600</v>
       </c>
       <c r="H46" s="12" t="n">
-        <v>585</v>
+        <v>540</v>
       </c>
       <c r="I46" s="12" t="n">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>микролот</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Колумбия Лили Роза Варгас Морено Чирозо Катуа </t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="inlineStr"/>
+      <c r="D47" s="12" t="n">
+        <v>2832.5</v>
+      </c>
+      <c r="E47" s="12" t="n">
+        <v>2550</v>
+      </c>
+      <c r="F47" s="12" t="n">
+        <v>2270</v>
+      </c>
+      <c r="G47" s="12" t="n">
+        <v>645</v>
+      </c>
+      <c r="H47" s="12" t="n">
+        <v>580.5</v>
+      </c>
+      <c r="I47" s="12" t="n">
         <v>520</v>
-      </c>
-    </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="13" t="inlineStr">
-        <is>
-          <t>микролот</t>
-        </is>
-      </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Колумбия Лили Роза Варгас Морено Чирозо Катуа </t>
-        </is>
-      </c>
-      <c r="C47" s="14" t="inlineStr"/>
-      <c r="D47" s="15" t="n">
-        <v>3102.5</v>
-      </c>
-      <c r="E47" s="15" t="n">
-        <v>2795</v>
-      </c>
-      <c r="F47" s="15" t="n">
-        <v>2485</v>
-      </c>
-      <c r="G47" s="15" t="n">
-        <v>700</v>
-      </c>
-      <c r="H47" s="15" t="n">
-        <v>630</v>
-      </c>
-      <c r="I47" s="15" t="n">
-        <v>560</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>🆕 микролот</t>
+          <t>микролот</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
@@ -2150,28 +2150,28 @@
         </is>
       </c>
       <c r="D48" s="12" t="n">
-        <v>5922.5</v>
+        <v>5397.5</v>
       </c>
       <c r="E48" s="12" t="n">
-        <v>5335</v>
+        <v>4860</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>4740</v>
+        <v>4320</v>
       </c>
       <c r="G48" s="12" t="n">
-        <v>1265</v>
+        <v>1160</v>
       </c>
       <c r="H48" s="12" t="n">
-        <v>1138.5</v>
+        <v>1044</v>
       </c>
       <c r="I48" s="12" t="n">
-        <v>1015</v>
+        <v>930</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>🆕 микролот</t>
+          <t>микролот</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
@@ -2185,115 +2185,115 @@
         </is>
       </c>
       <c r="D49" s="12" t="n">
-        <v>4842.5</v>
+        <v>4415</v>
       </c>
       <c r="E49" s="12" t="n">
-        <v>4360</v>
+        <v>3975</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>3875</v>
+        <v>3535</v>
       </c>
       <c r="G49" s="12" t="n">
-        <v>1050</v>
+        <v>965</v>
       </c>
       <c r="H49" s="12" t="n">
-        <v>945</v>
+        <v>868.5</v>
       </c>
       <c r="I49" s="12" t="n">
-        <v>840</v>
+        <v>775</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="13" t="inlineStr">
+      <c r="A50" s="10" t="inlineStr">
         <is>
           <t>микролот</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
+      <c r="B50" s="10" t="inlineStr">
         <is>
           <t>Колумбия Хиросос мытый</t>
         </is>
       </c>
-      <c r="C50" s="14" t="inlineStr"/>
-      <c r="D50" s="15" t="n">
-        <v>2547.5</v>
-      </c>
-      <c r="E50" s="15" t="n">
-        <v>2295</v>
-      </c>
-      <c r="F50" s="15" t="n">
-        <v>2040</v>
-      </c>
-      <c r="G50" s="15" t="n">
-        <v>590</v>
-      </c>
-      <c r="H50" s="15" t="n">
-        <v>531</v>
-      </c>
-      <c r="I50" s="15" t="n">
-        <v>475</v>
+      <c r="C50" s="11" t="inlineStr"/>
+      <c r="D50" s="12" t="n">
+        <v>2330</v>
+      </c>
+      <c r="E50" s="12" t="n">
+        <v>2100</v>
+      </c>
+      <c r="F50" s="12" t="n">
+        <v>1865</v>
+      </c>
+      <c r="G50" s="12" t="n">
+        <v>545</v>
+      </c>
+      <c r="H50" s="12" t="n">
+        <v>490.5</v>
+      </c>
+      <c r="I50" s="12" t="n">
+        <v>440</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="13" t="inlineStr">
+      <c r="A51" s="10" t="inlineStr">
         <is>
           <t>микролот</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
+      <c r="B51" s="10" t="inlineStr">
         <is>
           <t>КолумбияХайро Асрило инфьюз Маракуйя</t>
         </is>
       </c>
-      <c r="C51" s="14" t="inlineStr"/>
-      <c r="D51" s="15" t="n">
-        <v>4925</v>
-      </c>
-      <c r="E51" s="15" t="n">
-        <v>4435</v>
-      </c>
-      <c r="F51" s="15" t="n">
-        <v>3940</v>
-      </c>
-      <c r="G51" s="15" t="n">
-        <v>1065</v>
-      </c>
-      <c r="H51" s="15" t="n">
-        <v>958.5</v>
-      </c>
-      <c r="I51" s="15" t="n">
-        <v>855</v>
+      <c r="C51" s="11" t="inlineStr"/>
+      <c r="D51" s="12" t="n">
+        <v>4490</v>
+      </c>
+      <c r="E51" s="12" t="n">
+        <v>4045</v>
+      </c>
+      <c r="F51" s="12" t="n">
+        <v>3595</v>
+      </c>
+      <c r="G51" s="12" t="n">
+        <v>980</v>
+      </c>
+      <c r="H51" s="12" t="n">
+        <v>882</v>
+      </c>
+      <c r="I51" s="12" t="n">
+        <v>785</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="13" t="inlineStr">
+      <c r="A52" s="10" t="inlineStr">
         <is>
           <t>микролот</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
+      <c r="B52" s="10" t="inlineStr">
         <is>
           <t>Руанада Нямашеки хилс сухой</t>
         </is>
       </c>
-      <c r="C52" s="14" t="inlineStr"/>
-      <c r="D52" s="15" t="n">
-        <v>2862.5</v>
-      </c>
-      <c r="E52" s="15" t="n">
-        <v>2580</v>
-      </c>
-      <c r="F52" s="15" t="n">
-        <v>2290</v>
-      </c>
-      <c r="G52" s="15" t="n">
-        <v>655</v>
-      </c>
-      <c r="H52" s="15" t="n">
-        <v>589.5</v>
-      </c>
-      <c r="I52" s="15" t="n">
-        <v>525</v>
+      <c r="C52" s="11" t="inlineStr"/>
+      <c r="D52" s="12" t="n">
+        <v>2615</v>
+      </c>
+      <c r="E52" s="12" t="n">
+        <v>2355</v>
+      </c>
+      <c r="F52" s="12" t="n">
+        <v>2095</v>
+      </c>
+      <c r="G52" s="12" t="n">
+        <v>605</v>
+      </c>
+      <c r="H52" s="12" t="n">
+        <v>544.5</v>
+      </c>
+      <c r="I52" s="12" t="n">
+        <v>485</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bishop: Auto stock sync from 1C: stock updates 2
</commit_message>
<xml_diff>
--- a/tma_static/data/Roastberry_Прайс_2026.xlsx
+++ b/tma_static/data/Roastberry_Прайс_2026.xlsx
@@ -79,12 +79,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -143,22 +143,22 @@
     <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -550,86 +550,62 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Действует с 01.07.2026 · обновлено 29.06.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
           <t>Скидки: −10% от 10 кг · −20% от 25 кг</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Тип</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Название</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Обжарка</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Базовый (1 кг)</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>от 10 кг</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>от 25 кг</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Базовый (200 г)</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>от 10 кг</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>от 25 кг</t>
         </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>blend Es</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>CLASSICA  #1</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="6" t="n">
-        <v>1875</v>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>1690</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>1500</v>
-      </c>
-      <c r="G4" s="6" t="n">
-        <v>405</v>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>364.5</v>
-      </c>
-      <c r="I4" s="6" t="n">
-        <v>324</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -640,7 +616,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>БИТТЕР</t>
+          <t>CLASSICA #1</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -649,22 +625,22 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>1815</v>
+        <v>1875</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>1635</v>
+        <v>1690</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>1455</v>
+        <v>1500</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>395</v>
+        <v>405</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>355.5</v>
+        <v>364.5</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>316</v>
+        <v>324</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
@@ -675,7 +651,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>ВЕНЕЦИЯ</t>
+          <t>БИТТЕР</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -684,22 +660,22 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>1910</v>
+        <v>1815</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>1720</v>
+        <v>1635</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>1530</v>
+        <v>1455</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>410</v>
+        <v>395</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>369</v>
+        <v>355.5</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>328</v>
+        <v>316</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
@@ -710,7 +686,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>ХАНИ</t>
+          <t>ВЕНЕЦИЯ</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -740,17 +716,17 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>blend F</t>
+          <t>blend Es</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>ЛУНГО</t>
+          <t>ХАНИ</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>BF</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="D8" s="6" t="n">
@@ -773,38 +749,38 @@
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>моносорт</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Бразилия САН РАФАЕЛЬ сухой</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="n">
-        <v>1960</v>
-      </c>
-      <c r="E9" s="9" t="n">
-        <v>1765</v>
-      </c>
-      <c r="F9" s="9" t="n">
-        <v>1570</v>
-      </c>
-      <c r="G9" s="9" t="n">
-        <v>420</v>
-      </c>
-      <c r="H9" s="9" t="n">
-        <v>378</v>
-      </c>
-      <c r="I9" s="9" t="n">
-        <v>336</v>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>blend F</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>ЛУНГО</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>1910</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>1720</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>1530</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>410</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>369</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>328</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -815,31 +791,31 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Бразилия Серрадо желтый бурбон сухой</t>
+          <t>Бразилия Сан Рафаель</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>2005</v>
+        <v>1960</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>1805</v>
+        <v>1765</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>1605</v>
+        <v>1570</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>387</v>
+        <v>378</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>344</v>
+        <v>336</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
@@ -850,31 +826,31 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Бразилия Серрадо сухой/Бразилия Дарк </t>
+          <t>Бразилия Серрадо Желтый бурбон</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D11" s="9" t="n">
-        <v>1910</v>
+        <v>2005</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>1720</v>
+        <v>1805</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>1530</v>
+        <v>1605</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>410</v>
+        <v>430</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>369</v>
+        <v>387</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>328</v>
+        <v>344</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
@@ -885,31 +861,31 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Вьетнам Блю Шонла</t>
+          <t>Бразилия Серрадо Дарк</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>F E</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D12" s="9" t="n">
-        <v>2015</v>
+        <v>1910</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>1815</v>
+        <v>1720</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>1615</v>
+        <v>1530</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>435</v>
+        <v>410</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>391.5</v>
+        <v>369</v>
       </c>
       <c r="I12" s="9" t="n">
-        <v>348</v>
+        <v>328</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
@@ -920,7 +896,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Гватемалла Грок</t>
+          <t>Вьетнам Блю Шонла</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
@@ -929,22 +905,22 @@
         </is>
       </c>
       <c r="D13" s="9" t="n">
-        <v>2005</v>
+        <v>2015</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>1805</v>
+        <v>1815</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>1605</v>
+        <v>1615</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>430</v>
+        <v>435</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>387</v>
+        <v>391.5</v>
       </c>
       <c r="I13" s="9" t="n">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
@@ -955,31 +931,31 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Гватемалла Декаф</t>
+          <t>Гватемала Уэуэтенанго</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F E</t>
         </is>
       </c>
       <c r="D14" s="9" t="n">
-        <v>2295</v>
+        <v>2005</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>2070</v>
+        <v>1805</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>1840</v>
+        <v>1605</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>490</v>
+        <v>430</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>441</v>
+        <v>387</v>
       </c>
       <c r="I14" s="9" t="n">
-        <v>392</v>
+        <v>344</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -990,7 +966,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Гондурас Сан Николас мытый</t>
+          <t>Гватемала Декаф</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -999,22 +975,22 @@
         </is>
       </c>
       <c r="D15" s="9" t="n">
-        <v>2055</v>
+        <v>2295</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>1850</v>
+        <v>2070</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>1645</v>
+        <v>1840</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>440</v>
+        <v>490</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>396</v>
+        <v>441</v>
       </c>
       <c r="I15" s="9" t="n">
-        <v>352</v>
+        <v>392</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
@@ -1025,31 +1001,31 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Кения АА мытый</t>
+          <t>Гондурас Сан Николас</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D16" s="9" t="n">
-        <v>2440</v>
+        <v>2055</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>2200</v>
+        <v>1850</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>1955</v>
+        <v>1645</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>520</v>
+        <v>440</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>468</v>
+        <v>396</v>
       </c>
       <c r="I16" s="9" t="n">
-        <v>416</v>
+        <v>352</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
@@ -1060,31 +1036,31 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Кения Центральный провинции АБ мытый</t>
+          <t>Кения АА</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>E F</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D17" s="9" t="n">
-        <v>2345</v>
+        <v>2440</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>2115</v>
+        <v>2200</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>1880</v>
+        <v>1955</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>500</v>
+        <v>520</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>450</v>
+        <v>468</v>
       </c>
       <c r="I17" s="9" t="n">
-        <v>400</v>
+        <v>416</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
@@ -1095,31 +1071,31 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Китай Симао Гр.1 мытый</t>
+          <t>Кения АБ Центральная провинция</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>F E</t>
+          <t>E F</t>
         </is>
       </c>
       <c r="D18" s="9" t="n">
-        <v>1910</v>
+        <v>2345</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>1720</v>
+        <v>2115</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>1530</v>
+        <v>1880</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>410</v>
+        <v>500</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>369</v>
+        <v>450</v>
       </c>
       <c r="I18" s="9" t="n">
-        <v>328</v>
+        <v>400</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
@@ -1130,31 +1106,31 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Колумбия Андино мытый</t>
+          <t>Китай Симао Гр.1</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>E F</t>
+          <t>F E</t>
         </is>
       </c>
       <c r="D19" s="9" t="n">
-        <v>2055</v>
+        <v>1910</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>1850</v>
+        <v>1720</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>1645</v>
+        <v>1530</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>440</v>
+        <v>410</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>396</v>
+        <v>369</v>
       </c>
       <c r="I19" s="9" t="n">
-        <v>352</v>
+        <v>328</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -1165,31 +1141,31 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Коста-Рика Тарразу мытый</t>
+          <t>Колумбия Андино</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>E F</t>
         </is>
       </c>
       <c r="D20" s="9" t="n">
-        <v>2120</v>
+        <v>2055</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>1910</v>
+        <v>1850</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>1700</v>
+        <v>1645</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>455</v>
+        <v>440</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>409.5</v>
+        <v>396</v>
       </c>
       <c r="I20" s="9" t="n">
-        <v>364</v>
+        <v>352</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
@@ -1200,7 +1176,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Никарагуа Марагаджип мытый</t>
+          <t>Коста-Рика Тарразу</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
@@ -1209,22 +1185,22 @@
         </is>
       </c>
       <c r="D21" s="9" t="n">
-        <v>2390</v>
+        <v>2120</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>2155</v>
+        <v>1910</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>1915</v>
+        <v>1700</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>510</v>
+        <v>455</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>459</v>
+        <v>409.5</v>
       </c>
       <c r="I21" s="9" t="n">
-        <v>408</v>
+        <v>364</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
@@ -1235,7 +1211,7 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Перу Гр.1</t>
+          <t>Никарагуа Марагаджип</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
@@ -1244,22 +1220,22 @@
         </is>
       </c>
       <c r="D22" s="9" t="n">
-        <v>2105</v>
+        <v>2390</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>1895</v>
+        <v>2155</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>1685</v>
+        <v>1915</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>450</v>
+        <v>510</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>405</v>
+        <v>459</v>
       </c>
       <c r="I22" s="9" t="n">
-        <v>360</v>
+        <v>408</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
@@ -1270,31 +1246,31 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Перу Монте Верде сухой</t>
+          <t>Перу гр.1</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D23" s="9" t="n">
-        <v>2460</v>
+        <v>2105</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>2215</v>
+        <v>1895</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>1970</v>
+        <v>1685</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>520</v>
+        <v>450</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>468</v>
+        <v>405</v>
       </c>
       <c r="I23" s="9" t="n">
-        <v>416</v>
+        <v>360</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
@@ -1305,7 +1281,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Руанада Мутителли 15+</t>
+          <t>Перу Монте Верде</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
@@ -1314,22 +1290,22 @@
         </is>
       </c>
       <c r="D24" s="9" t="n">
-        <v>2105</v>
+        <v>2460</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>1895</v>
+        <v>2215</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>1685</v>
+        <v>1970</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>405</v>
+        <v>468</v>
       </c>
       <c r="I24" s="9" t="n">
-        <v>360</v>
+        <v>416</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
@@ -1340,7 +1316,7 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Танзания АА</t>
+          <t>Руанда Мутетели</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
@@ -1349,22 +1325,22 @@
         </is>
       </c>
       <c r="D25" s="9" t="n">
-        <v>2200</v>
+        <v>2105</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>1980</v>
+        <v>1895</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>1760</v>
+        <v>1685</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>470</v>
+        <v>450</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>423</v>
+        <v>405</v>
       </c>
       <c r="I25" s="9" t="n">
-        <v>376</v>
+        <v>360</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
@@ -1375,31 +1351,31 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Уганда Вугар Элгон мытый </t>
+          <t>Танзания АА</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D26" s="9" t="n">
-        <v>1960</v>
+        <v>2200</v>
       </c>
       <c r="E26" s="9" t="n">
-        <v>1765</v>
+        <v>1980</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>1570</v>
+        <v>1760</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>420</v>
+        <v>470</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>378</v>
+        <v>423</v>
       </c>
       <c r="I26" s="9" t="n">
-        <v>336</v>
+        <v>376</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
@@ -1410,7 +1386,7 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Уганда Рувензор сухой</t>
+          <t>Уганда Вугар Элгон</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
@@ -1419,22 +1395,22 @@
         </is>
       </c>
       <c r="D27" s="9" t="n">
-        <v>1910</v>
+        <v>1960</v>
       </c>
       <c r="E27" s="9" t="n">
-        <v>1720</v>
+        <v>1765</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>1530</v>
+        <v>1570</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>410</v>
+        <v>420</v>
       </c>
       <c r="H27" s="9" t="n">
-        <v>369</v>
+        <v>378</v>
       </c>
       <c r="I27" s="9" t="n">
-        <v>328</v>
+        <v>336</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
@@ -1445,7 +1421,7 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Эфиопия Арича Гр.3 сухой </t>
+          <t>Уганда Рувензор</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
@@ -1454,22 +1430,22 @@
         </is>
       </c>
       <c r="D28" s="9" t="n">
-        <v>2055</v>
+        <v>1910</v>
       </c>
       <c r="E28" s="9" t="n">
-        <v>1850</v>
+        <v>1720</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>1645</v>
+        <v>1530</v>
       </c>
       <c r="G28" s="9" t="n">
-        <v>440</v>
+        <v>410</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>396</v>
+        <v>369</v>
       </c>
       <c r="I28" s="9" t="n">
-        <v>352</v>
+        <v>328</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
@@ -1480,7 +1456,7 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Эфиопия Иргач Гр.4 ТОП сухой /Эфиопи Милк (темн)</t>
+          <t>Эфиопия Арича гр.3</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
@@ -1489,22 +1465,22 @@
         </is>
       </c>
       <c r="D29" s="9" t="n">
-        <v>1910</v>
+        <v>2055</v>
       </c>
       <c r="E29" s="9" t="n">
-        <v>1720</v>
+        <v>1850</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>1530</v>
+        <v>1645</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>410</v>
+        <v>440</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>369</v>
+        <v>396</v>
       </c>
       <c r="I29" s="9" t="n">
-        <v>328</v>
+        <v>352</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
@@ -1515,31 +1491,31 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Эфиопия Лиму Гр.2 мытый</t>
+          <t>Эфопия Иргачиф Гр.4</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D30" s="9" t="n">
-        <v>2005</v>
+        <v>1910</v>
       </c>
       <c r="E30" s="9" t="n">
-        <v>1805</v>
+        <v>1720</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>1605</v>
+        <v>1530</v>
       </c>
       <c r="G30" s="9" t="n">
-        <v>430</v>
+        <v>410</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>387</v>
+        <v>369</v>
       </c>
       <c r="I30" s="9" t="n">
-        <v>344</v>
+        <v>328</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
@@ -1550,12 +1526,12 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Эфиопия Сидамо Гр.2 Гуджи мытый</t>
+          <t>Эфиопия Лиму Гр.2</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>E F</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D31" s="9" t="n">
@@ -1578,434 +1554,434 @@
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>микролот • BLACK</t>
-        </is>
-      </c>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>Колумбия Клаудиа Колменарес Гейша мытый</t>
-        </is>
-      </c>
-      <c r="C32" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D32" s="12" t="n">
-        <v>3192.5</v>
-      </c>
-      <c r="E32" s="12" t="n">
-        <v>2875</v>
-      </c>
-      <c r="F32" s="12" t="n">
-        <v>2555</v>
-      </c>
-      <c r="G32" s="12" t="n">
-        <v>720</v>
-      </c>
-      <c r="H32" s="12" t="n">
-        <v>648</v>
-      </c>
-      <c r="I32" s="12" t="n">
-        <v>580</v>
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>моносорт</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Эфиопия Сидамо Гр.2 Гуджи</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>E F</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="n">
+        <v>2005</v>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>1805</v>
+      </c>
+      <c r="F32" s="9" t="n">
+        <v>1605</v>
+      </c>
+      <c r="G32" s="9" t="n">
+        <v>430</v>
+      </c>
+      <c r="H32" s="9" t="n">
+        <v>387</v>
+      </c>
+      <c r="I32" s="9" t="n">
+        <v>344</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
         <is>
+          <t>NEW микролот • BLACK</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Кения Маакиоу Пиберри</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="n">
+        <v>2705</v>
+      </c>
+      <c r="E33" s="12" t="n">
+        <v>2435</v>
+      </c>
+      <c r="F33" s="12" t="n">
+        <v>2165</v>
+      </c>
+      <c r="G33" s="12" t="n">
+        <v>620</v>
+      </c>
+      <c r="H33" s="12" t="n">
+        <v>558</v>
+      </c>
+      <c r="I33" s="12" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t>Эфиопия Иргач Адада гр.1 сухой</t>
-        </is>
-      </c>
-      <c r="C33" s="11" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>Колумбия Кастильо</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D33" s="12" t="n">
+      <c r="D34" s="15" t="n">
+        <v>2600</v>
+      </c>
+      <c r="E34" s="15" t="n">
+        <v>2340</v>
+      </c>
+      <c r="F34" s="15" t="n">
+        <v>2080</v>
+      </c>
+      <c r="G34" s="15" t="n">
+        <v>600</v>
+      </c>
+      <c r="H34" s="15" t="n">
+        <v>540</v>
+      </c>
+      <c r="I34" s="15" t="n">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BLACK</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Колумбия Клаудиа Колменарес</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="n">
+        <v>3192.5</v>
+      </c>
+      <c r="E35" s="15" t="n">
+        <v>2875</v>
+      </c>
+      <c r="F35" s="15" t="n">
+        <v>2555</v>
+      </c>
+      <c r="G35" s="15" t="n">
+        <v>720</v>
+      </c>
+      <c r="H35" s="15" t="n">
+        <v>648</v>
+      </c>
+      <c r="I35" s="15" t="n">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BLACK</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Колумбия Лили Роза Варгас Морено</t>
+        </is>
+      </c>
+      <c r="C36" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D36" s="15" t="n">
+        <v>2832.5</v>
+      </c>
+      <c r="E36" s="15" t="n">
+        <v>2550</v>
+      </c>
+      <c r="F36" s="15" t="n">
+        <v>2270</v>
+      </c>
+      <c r="G36" s="15" t="n">
+        <v>645</v>
+      </c>
+      <c r="H36" s="15" t="n">
+        <v>580.5</v>
+      </c>
+      <c r="I36" s="15" t="n">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BLACK</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Колумбия Хиросос</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="n">
+        <v>2330</v>
+      </c>
+      <c r="E37" s="15" t="n">
+        <v>2100</v>
+      </c>
+      <c r="F37" s="15" t="n">
+        <v>1865</v>
+      </c>
+      <c r="G37" s="15" t="n">
+        <v>545</v>
+      </c>
+      <c r="H37" s="15" t="n">
+        <v>490.5</v>
+      </c>
+      <c r="I37" s="15" t="n">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BLACK</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Руанда Нямашеки Хиллс</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>E F</t>
+        </is>
+      </c>
+      <c r="D38" s="15" t="n">
+        <v>2615</v>
+      </c>
+      <c r="E38" s="15" t="n">
+        <v>2355</v>
+      </c>
+      <c r="F38" s="15" t="n">
+        <v>2095</v>
+      </c>
+      <c r="G38" s="15" t="n">
+        <v>605</v>
+      </c>
+      <c r="H38" s="15" t="n">
+        <v>544.5</v>
+      </c>
+      <c r="I38" s="15" t="n">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BLACK</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Эфиопия Ададо</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="n">
         <v>2187.5</v>
       </c>
-      <c r="E33" s="12" t="n">
+      <c r="E39" s="15" t="n">
         <v>1970</v>
       </c>
-      <c r="F33" s="12" t="n">
+      <c r="F39" s="15" t="n">
         <v>1750</v>
       </c>
-      <c r="G33" s="12" t="n">
+      <c r="G39" s="15" t="n">
         <v>520</v>
       </c>
-      <c r="H33" s="12" t="n">
+      <c r="H39" s="15" t="n">
         <v>468</v>
       </c>
-      <c r="I33" s="12" t="n">
+      <c r="I39" s="15" t="n">
         <v>420</v>
       </c>
     </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="10" t="inlineStr">
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="13" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B34" s="10" t="inlineStr">
-        <is>
-          <t>Эфиопия Иргач Билоя гр.2 сухой</t>
-        </is>
-      </c>
-      <c r="C34" s="11" t="inlineStr">
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>Эфиопия Белойя гр.2</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D34" s="12" t="n">
+      <c r="D40" s="15" t="n">
         <v>2045</v>
       </c>
-      <c r="E34" s="12" t="n">
+      <c r="E40" s="15" t="n">
         <v>1845</v>
       </c>
-      <c r="F34" s="12" t="n">
+      <c r="F40" s="15" t="n">
         <v>1640</v>
       </c>
-      <c r="G34" s="12" t="n">
+      <c r="G40" s="15" t="n">
         <v>490</v>
       </c>
-      <c r="H34" s="12" t="n">
+      <c r="H40" s="15" t="n">
         <v>441</v>
       </c>
-      <c r="I34" s="12" t="n">
+      <c r="I40" s="15" t="n">
         <v>395</v>
       </c>
     </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="10" t="inlineStr">
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="13" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B35" s="10" t="inlineStr">
-        <is>
-          <t>Эфиопия Иргач Челелекту мытый гр.1</t>
-        </is>
-      </c>
-      <c r="C35" s="11" t="inlineStr">
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>Эфиопия Челелекту гр.1</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D35" s="12" t="n">
+      <c r="D41" s="15" t="n">
         <v>2615</v>
       </c>
-      <c r="E35" s="12" t="n">
+      <c r="E41" s="15" t="n">
         <v>2355</v>
       </c>
-      <c r="F35" s="12" t="n">
+      <c r="F41" s="15" t="n">
         <v>2095</v>
       </c>
-      <c r="G35" s="12" t="n">
+      <c r="G41" s="15" t="n">
         <v>605</v>
       </c>
-      <c r="H35" s="12" t="n">
+      <c r="H41" s="15" t="n">
         <v>544.5</v>
       </c>
-      <c r="I35" s="12" t="n">
+      <c r="I41" s="15" t="n">
         <v>485</v>
       </c>
     </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="10" t="inlineStr">
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>Эфиопия Челчеле гр.1 сухой</t>
-        </is>
-      </c>
-      <c r="C36" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D36" s="12" t="n">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>Эфиопия Челчеле гр.1</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>E F</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="n">
         <v>2615</v>
       </c>
-      <c r="E36" s="12" t="n">
+      <c r="E42" s="15" t="n">
         <v>2355</v>
       </c>
-      <c r="F36" s="12" t="n">
+      <c r="F42" s="15" t="n">
         <v>2095</v>
       </c>
-      <c r="G36" s="12" t="n">
+      <c r="G42" s="15" t="n">
         <v>605</v>
       </c>
-      <c r="H36" s="12" t="n">
+      <c r="H42" s="15" t="n">
         <v>544.5</v>
       </c>
-      <c r="I36" s="12" t="n">
+      <c r="I42" s="15" t="n">
         <v>485</v>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="10" t="inlineStr">
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t>Бразилия SL28 Хани анаэроб.</t>
-        </is>
-      </c>
-      <c r="C37" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D37" s="12" t="n">
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>Бразилия SL28</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>E F</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="n">
         <v>3192.5</v>
       </c>
-      <c r="E37" s="12" t="n">
+      <c r="E43" s="15" t="n">
         <v>2875</v>
       </c>
-      <c r="F37" s="12" t="n">
+      <c r="F43" s="15" t="n">
         <v>2555</v>
       </c>
-      <c r="G37" s="12" t="n">
+      <c r="G43" s="15" t="n">
         <v>720</v>
       </c>
-      <c r="H37" s="12" t="n">
+      <c r="H43" s="15" t="n">
         <v>648</v>
       </c>
-      <c r="I37" s="12" t="n">
+      <c r="I43" s="15" t="n">
         <v>580</v>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="10" t="inlineStr">
-        <is>
-          <t>микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t>Бразилия Судан Руме анаэроб.</t>
-        </is>
-      </c>
-      <c r="C38" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D38" s="12" t="n">
-        <v>3192.5</v>
-      </c>
-      <c r="E38" s="12" t="n">
-        <v>2875</v>
-      </c>
-      <c r="F38" s="12" t="n">
-        <v>2555</v>
-      </c>
-      <c r="G38" s="12" t="n">
-        <v>720</v>
-      </c>
-      <c r="H38" s="12" t="n">
-        <v>648</v>
-      </c>
-      <c r="I38" s="12" t="n">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="10" t="inlineStr">
-        <is>
-          <t>микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B39" s="10" t="inlineStr">
-        <is>
-          <t>Бразилия Фазенда Лагуинья мундо анаэроб.</t>
-        </is>
-      </c>
-      <c r="C39" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D39" s="12" t="n">
-        <v>3192.5</v>
-      </c>
-      <c r="E39" s="12" t="n">
-        <v>2875</v>
-      </c>
-      <c r="F39" s="12" t="n">
-        <v>2555</v>
-      </c>
-      <c r="G39" s="12" t="n">
-        <v>720</v>
-      </c>
-      <c r="H39" s="12" t="n">
-        <v>648</v>
-      </c>
-      <c r="I39" s="12" t="n">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t>микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B40" s="10" t="inlineStr">
-        <is>
-          <t>Колумбия Гонзало Кормана Катура сухой</t>
-        </is>
-      </c>
-      <c r="C40" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D40" s="12" t="n">
-        <v>3192.5</v>
-      </c>
-      <c r="E40" s="12" t="n">
-        <v>2875</v>
-      </c>
-      <c r="F40" s="12" t="n">
-        <v>2555</v>
-      </c>
-      <c r="G40" s="12" t="n">
-        <v>720</v>
-      </c>
-      <c r="H40" s="12" t="n">
-        <v>648</v>
-      </c>
-      <c r="I40" s="12" t="n">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t>Колумбия Хайро Арсило сухой</t>
-        </is>
-      </c>
-      <c r="C41" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D41" s="12" t="n">
-        <v>2615</v>
-      </c>
-      <c r="E41" s="12" t="n">
-        <v>2355</v>
-      </c>
-      <c r="F41" s="12" t="n">
-        <v>2095</v>
-      </c>
-      <c r="G41" s="12" t="n">
-        <v>605</v>
-      </c>
-      <c r="H41" s="12" t="n">
-        <v>544.5</v>
-      </c>
-      <c r="I41" s="12" t="n">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="10" t="inlineStr">
-        <is>
-          <t>микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B42" s="10" t="inlineStr">
-        <is>
-          <t>Смесь Экваториальная</t>
-        </is>
-      </c>
-      <c r="C42" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D42" s="12" t="n">
-        <v>2765</v>
-      </c>
-      <c r="E42" s="12" t="n">
-        <v>2490</v>
-      </c>
-      <c r="F42" s="12" t="n">
-        <v>2215</v>
-      </c>
-      <c r="G42" s="12" t="n">
-        <v>635</v>
-      </c>
-      <c r="H42" s="12" t="n">
-        <v>571.5</v>
-      </c>
-      <c r="I42" s="12" t="n">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="10" t="inlineStr">
-        <is>
-          <t>микролот • BORЩ</t>
-        </is>
-      </c>
-      <c r="B43" s="10" t="inlineStr">
-        <is>
-          <t>Эфиопия Арича гр.1 сухой</t>
-        </is>
-      </c>
-      <c r="C43" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D43" s="12" t="n">
-        <v>2765</v>
-      </c>
-      <c r="E43" s="12" t="n">
-        <v>2490</v>
-      </c>
-      <c r="F43" s="12" t="n">
-        <v>2215</v>
-      </c>
-      <c r="G43" s="12" t="n">
-        <v>635</v>
-      </c>
-      <c r="H43" s="12" t="n">
-        <v>571.5</v>
-      </c>
-      <c r="I43" s="12" t="n">
-        <v>510</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>🆕 микролот</t>
+          <t>микролот • BORЩ</t>
         </is>
       </c>
       <c r="B44" s="13" t="inlineStr">
         <is>
-          <t>Кения КиаваМуруру нат.анаэроб.</t>
+          <t>Бразилия Судан Руме</t>
         </is>
       </c>
       <c r="C44" s="14" t="inlineStr">
@@ -2014,68 +1990,68 @@
         </is>
       </c>
       <c r="D44" s="15" t="n">
-        <v>3627.5</v>
+        <v>3192.5</v>
       </c>
       <c r="E44" s="15" t="n">
-        <v>3265</v>
+        <v>2875</v>
       </c>
       <c r="F44" s="15" t="n">
-        <v>2905</v>
+        <v>2555</v>
       </c>
       <c r="G44" s="15" t="n">
-        <v>805</v>
+        <v>720</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>724.5</v>
+        <v>648</v>
       </c>
       <c r="I44" s="15" t="n">
-        <v>645</v>
+        <v>580</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>🆕 микролот</t>
+          <t>микролот • BORЩ</t>
         </is>
       </c>
       <c r="B45" s="13" t="inlineStr">
         <is>
-          <t>Кения Маакиоу Пиберри</t>
+          <t>Бразилия Фазенда Лагуинья мундо</t>
         </is>
       </c>
       <c r="C45" s="14" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E F</t>
         </is>
       </c>
       <c r="D45" s="15" t="n">
-        <v>2705</v>
+        <v>3192.5</v>
       </c>
       <c r="E45" s="15" t="n">
-        <v>2435</v>
+        <v>2875</v>
       </c>
       <c r="F45" s="15" t="n">
-        <v>2165</v>
+        <v>2555</v>
       </c>
       <c r="G45" s="15" t="n">
-        <v>620</v>
+        <v>720</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>558</v>
+        <v>648</v>
       </c>
       <c r="I45" s="15" t="n">
-        <v>500</v>
+        <v>580</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>микролот</t>
+          <t>NEW микролот • BORЩ</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>Колумбия Кастильо</t>
+          <t>Кения КиаваМуруру</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
@@ -2084,221 +2060,238 @@
         </is>
       </c>
       <c r="D46" s="12" t="n">
-        <v>2600</v>
+        <v>3627.5</v>
       </c>
       <c r="E46" s="12" t="n">
-        <v>2340</v>
+        <v>3265</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>2080</v>
+        <v>2905</v>
       </c>
       <c r="G46" s="12" t="n">
-        <v>600</v>
+        <v>805</v>
       </c>
       <c r="H46" s="12" t="n">
-        <v>540</v>
+        <v>724.5</v>
       </c>
       <c r="I46" s="12" t="n">
-        <v>480</v>
+        <v>645</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="10" t="inlineStr">
-        <is>
-          <t>микролот</t>
-        </is>
-      </c>
-      <c r="B47" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Колумбия Лили Роза Варгас Морено Чирозо Катуа </t>
-        </is>
-      </c>
-      <c r="C47" s="11" t="inlineStr"/>
-      <c r="D47" s="12" t="n">
-        <v>2832.5</v>
-      </c>
-      <c r="E47" s="12" t="n">
-        <v>2550</v>
-      </c>
-      <c r="F47" s="12" t="n">
-        <v>2270</v>
-      </c>
-      <c r="G47" s="12" t="n">
-        <v>645</v>
-      </c>
-      <c r="H47" s="12" t="n">
-        <v>580.5</v>
-      </c>
-      <c r="I47" s="12" t="n">
-        <v>520</v>
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BORЩ</t>
+        </is>
+      </c>
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>Колумбия Гонзало Кармона</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="n">
+        <v>3192.5</v>
+      </c>
+      <c r="E47" s="15" t="n">
+        <v>2875</v>
+      </c>
+      <c r="F47" s="15" t="n">
+        <v>2555</v>
+      </c>
+      <c r="G47" s="15" t="n">
+        <v>720</v>
+      </c>
+      <c r="H47" s="15" t="n">
+        <v>648</v>
+      </c>
+      <c r="I47" s="15" t="n">
+        <v>580</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="10" t="inlineStr">
-        <is>
-          <t>микролот</t>
-        </is>
-      </c>
-      <c r="B48" s="10" t="inlineStr">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BORЩ</t>
+        </is>
+      </c>
+      <c r="B48" s="13" t="inlineStr">
         <is>
           <t>Колумбия Маракуйя</t>
         </is>
       </c>
-      <c r="C48" s="11" t="inlineStr">
+      <c r="C48" s="14" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D48" s="12" t="n">
+      <c r="D48" s="15" t="n">
         <v>5397.5</v>
       </c>
-      <c r="E48" s="12" t="n">
+      <c r="E48" s="15" t="n">
         <v>4860</v>
       </c>
-      <c r="F48" s="12" t="n">
+      <c r="F48" s="15" t="n">
         <v>4320</v>
       </c>
-      <c r="G48" s="12" t="n">
+      <c r="G48" s="15" t="n">
         <v>1160</v>
       </c>
-      <c r="H48" s="12" t="n">
+      <c r="H48" s="15" t="n">
         <v>1044</v>
       </c>
-      <c r="I48" s="12" t="n">
+      <c r="I48" s="15" t="n">
         <v>930</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="10" t="inlineStr">
-        <is>
-          <t>микролот</t>
-        </is>
-      </c>
-      <c r="B49" s="10" t="inlineStr">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BORЩ</t>
+        </is>
+      </c>
+      <c r="B49" s="13" t="inlineStr">
         <is>
           <t>Колумбия Пачамама</t>
         </is>
       </c>
-      <c r="C49" s="11" t="inlineStr">
+      <c r="C49" s="14" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D49" s="12" t="n">
+      <c r="D49" s="15" t="n">
         <v>4415</v>
       </c>
-      <c r="E49" s="12" t="n">
+      <c r="E49" s="15" t="n">
         <v>3975</v>
       </c>
-      <c r="F49" s="12" t="n">
+      <c r="F49" s="15" t="n">
         <v>3535</v>
       </c>
-      <c r="G49" s="12" t="n">
+      <c r="G49" s="15" t="n">
         <v>965</v>
       </c>
-      <c r="H49" s="12" t="n">
+      <c r="H49" s="15" t="n">
         <v>868.5</v>
       </c>
-      <c r="I49" s="12" t="n">
+      <c r="I49" s="15" t="n">
         <v>775</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="10" t="inlineStr">
-        <is>
-          <t>микролот</t>
-        </is>
-      </c>
-      <c r="B50" s="10" t="inlineStr">
-        <is>
-          <t>Колумбия Хиросос мытый</t>
-        </is>
-      </c>
-      <c r="C50" s="11" t="inlineStr"/>
-      <c r="D50" s="12" t="n">
-        <v>2330</v>
-      </c>
-      <c r="E50" s="12" t="n">
-        <v>2100</v>
-      </c>
-      <c r="F50" s="12" t="n">
-        <v>1865</v>
-      </c>
-      <c r="G50" s="12" t="n">
-        <v>545</v>
-      </c>
-      <c r="H50" s="12" t="n">
-        <v>490.5</v>
-      </c>
-      <c r="I50" s="12" t="n">
-        <v>440</v>
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BORЩ</t>
+        </is>
+      </c>
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>Колумбия Хайро Арсила</t>
+        </is>
+      </c>
+      <c r="C50" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D50" s="15" t="n">
+        <v>2615</v>
+      </c>
+      <c r="E50" s="15" t="n">
+        <v>2355</v>
+      </c>
+      <c r="F50" s="15" t="n">
+        <v>2095</v>
+      </c>
+      <c r="G50" s="15" t="n">
+        <v>605</v>
+      </c>
+      <c r="H50" s="15" t="n">
+        <v>544.5</v>
+      </c>
+      <c r="I50" s="15" t="n">
+        <v>485</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="10" t="inlineStr">
-        <is>
-          <t>микролот</t>
-        </is>
-      </c>
-      <c r="B51" s="10" t="inlineStr">
-        <is>
-          <t>КолумбияХайро Асрило инфьюз Маракуйя</t>
-        </is>
-      </c>
-      <c r="C51" s="11" t="inlineStr"/>
-      <c r="D51" s="12" t="n">
-        <v>4490</v>
-      </c>
-      <c r="E51" s="12" t="n">
-        <v>4045</v>
-      </c>
-      <c r="F51" s="12" t="n">
-        <v>3595</v>
-      </c>
-      <c r="G51" s="12" t="n">
-        <v>980</v>
-      </c>
-      <c r="H51" s="12" t="n">
-        <v>882</v>
-      </c>
-      <c r="I51" s="12" t="n">
-        <v>785</v>
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BORЩ</t>
+        </is>
+      </c>
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>Экваториальный блэнд</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D51" s="15" t="n">
+        <v>2765</v>
+      </c>
+      <c r="E51" s="15" t="n">
+        <v>2490</v>
+      </c>
+      <c r="F51" s="15" t="n">
+        <v>2215</v>
+      </c>
+      <c r="G51" s="15" t="n">
+        <v>635</v>
+      </c>
+      <c r="H51" s="15" t="n">
+        <v>571.5</v>
+      </c>
+      <c r="I51" s="15" t="n">
+        <v>510</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="10" t="inlineStr">
-        <is>
-          <t>микролот</t>
-        </is>
-      </c>
-      <c r="B52" s="10" t="inlineStr">
-        <is>
-          <t>Руанада Нямашеки хилс сухой</t>
-        </is>
-      </c>
-      <c r="C52" s="11" t="inlineStr"/>
-      <c r="D52" s="12" t="n">
-        <v>2615</v>
-      </c>
-      <c r="E52" s="12" t="n">
-        <v>2355</v>
-      </c>
-      <c r="F52" s="12" t="n">
-        <v>2095</v>
-      </c>
-      <c r="G52" s="12" t="n">
-        <v>605</v>
-      </c>
-      <c r="H52" s="12" t="n">
-        <v>544.5</v>
-      </c>
-      <c r="I52" s="12" t="n">
-        <v>485</v>
+      <c r="A52" s="13" t="inlineStr">
+        <is>
+          <t>микролот • BORЩ</t>
+        </is>
+      </c>
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>Эфиопия Арича гр.1</t>
+        </is>
+      </c>
+      <c r="C52" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D52" s="15" t="n">
+        <v>2765</v>
+      </c>
+      <c r="E52" s="15" t="n">
+        <v>2490</v>
+      </c>
+      <c r="F52" s="15" t="n">
+        <v>2215</v>
+      </c>
+      <c r="G52" s="15" t="n">
+        <v>635</v>
+      </c>
+      <c r="H52" s="15" t="n">
+        <v>571.5</v>
+      </c>
+      <c r="I52" s="15" t="n">
+        <v>510</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Bishop: Drip + Borshch photos update
</commit_message>
<xml_diff>
--- a/tma_static/data/Roastberry_Прайс_2026.xlsx
+++ b/tma_static/data/Roastberry_Прайс_2026.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Прайс 2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прайс 2026" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -79,12 +79,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -143,22 +143,22 @@
     <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -550,7 +550,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Действует с 01.07.2026 · обновлено 30.06.2026</t>
+          <t>Действует с 01.07.2026 · обновлено 07.07.2026</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>NEW микролот • BLACK</t>
+          <t>микролот • BLACK</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
@@ -1624,429 +1624,429 @@
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="A34" s="10" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>Колумбия Кастильо</t>
         </is>
       </c>
-      <c r="C34" s="14" t="inlineStr">
+      <c r="C34" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D34" s="15" t="n">
+      <c r="D34" s="12" t="n">
         <v>2847.5</v>
       </c>
-      <c r="E34" s="15" t="n">
+      <c r="E34" s="12" t="n">
         <v>2565</v>
       </c>
-      <c r="F34" s="15" t="n">
+      <c r="F34" s="12" t="n">
         <v>2280</v>
       </c>
-      <c r="G34" s="15" t="n">
+      <c r="G34" s="12" t="n">
         <v>650</v>
       </c>
-      <c r="H34" s="15" t="n">
+      <c r="H34" s="12" t="n">
         <v>585</v>
       </c>
-      <c r="I34" s="15" t="n">
+      <c r="I34" s="12" t="n">
         <v>520</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="13" t="inlineStr">
+      <c r="A35" s="10" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="10" t="inlineStr">
         <is>
           <t>Колумбия Клаудиа Колменарес</t>
         </is>
       </c>
-      <c r="C35" s="14" t="inlineStr">
+      <c r="C35" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D35" s="15" t="n">
+      <c r="D35" s="12" t="n">
         <v>3500</v>
       </c>
-      <c r="E35" s="15" t="n">
+      <c r="E35" s="12" t="n">
         <v>3150</v>
       </c>
-      <c r="F35" s="15" t="n">
+      <c r="F35" s="12" t="n">
         <v>2800</v>
       </c>
-      <c r="G35" s="15" t="n">
+      <c r="G35" s="12" t="n">
         <v>780</v>
       </c>
-      <c r="H35" s="15" t="n">
+      <c r="H35" s="12" t="n">
         <v>702</v>
       </c>
-      <c r="I35" s="15" t="n">
+      <c r="I35" s="12" t="n">
         <v>625</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="13" t="inlineStr">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>Колумбия Лили Роза Варгас Морено</t>
         </is>
       </c>
-      <c r="C36" s="14" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D36" s="15" t="n">
+      <c r="D36" s="12" t="n">
         <v>3102.5</v>
       </c>
-      <c r="E36" s="15" t="n">
+      <c r="E36" s="12" t="n">
         <v>2795</v>
       </c>
-      <c r="F36" s="15" t="n">
+      <c r="F36" s="12" t="n">
         <v>2485</v>
       </c>
-      <c r="G36" s="15" t="n">
+      <c r="G36" s="12" t="n">
         <v>700</v>
       </c>
-      <c r="H36" s="15" t="n">
+      <c r="H36" s="12" t="n">
         <v>630</v>
       </c>
-      <c r="I36" s="15" t="n">
+      <c r="I36" s="12" t="n">
         <v>560</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="A37" s="10" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B37" s="13" t="inlineStr">
+      <c r="B37" s="10" t="inlineStr">
         <is>
           <t>Колумбия Хиросос</t>
         </is>
       </c>
-      <c r="C37" s="14" t="inlineStr">
+      <c r="C37" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D37" s="15" t="n">
+      <c r="D37" s="12" t="n">
         <v>2547.5</v>
       </c>
-      <c r="E37" s="15" t="n">
+      <c r="E37" s="12" t="n">
         <v>2295</v>
       </c>
-      <c r="F37" s="15" t="n">
+      <c r="F37" s="12" t="n">
         <v>2040</v>
       </c>
-      <c r="G37" s="15" t="n">
+      <c r="G37" s="12" t="n">
         <v>590</v>
       </c>
-      <c r="H37" s="15" t="n">
+      <c r="H37" s="12" t="n">
         <v>531</v>
       </c>
-      <c r="I37" s="15" t="n">
+      <c r="I37" s="12" t="n">
         <v>475</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="A38" s="10" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
+      <c r="B38" s="10" t="inlineStr">
         <is>
           <t>Руанда Нямашеки Хиллс</t>
         </is>
       </c>
-      <c r="C38" s="14" t="inlineStr">
+      <c r="C38" s="11" t="inlineStr">
         <is>
           <t>E F</t>
         </is>
       </c>
-      <c r="D38" s="15" t="n">
+      <c r="D38" s="12" t="n">
         <v>2862.5</v>
       </c>
-      <c r="E38" s="15" t="n">
+      <c r="E38" s="12" t="n">
         <v>2580</v>
       </c>
-      <c r="F38" s="15" t="n">
+      <c r="F38" s="12" t="n">
         <v>2290</v>
       </c>
-      <c r="G38" s="15" t="n">
+      <c r="G38" s="12" t="n">
         <v>655</v>
       </c>
-      <c r="H38" s="15" t="n">
+      <c r="H38" s="12" t="n">
         <v>589.5</v>
       </c>
-      <c r="I38" s="15" t="n">
+      <c r="I38" s="12" t="n">
         <v>525</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="A39" s="10" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
+      <c r="B39" s="10" t="inlineStr">
         <is>
           <t>Эфиопия Ададо</t>
         </is>
       </c>
-      <c r="C39" s="14" t="inlineStr">
+      <c r="C39" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D39" s="15" t="n">
+      <c r="D39" s="12" t="n">
         <v>2390</v>
       </c>
-      <c r="E39" s="15" t="n">
+      <c r="E39" s="12" t="n">
         <v>2155</v>
       </c>
-      <c r="F39" s="15" t="n">
+      <c r="F39" s="12" t="n">
         <v>1915</v>
       </c>
-      <c r="G39" s="15" t="n">
+      <c r="G39" s="12" t="n">
         <v>560</v>
       </c>
-      <c r="H39" s="15" t="n">
+      <c r="H39" s="12" t="n">
         <v>504</v>
       </c>
-      <c r="I39" s="15" t="n">
+      <c r="I39" s="12" t="n">
         <v>450</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="13" t="inlineStr">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
+      <c r="B40" s="10" t="inlineStr">
         <is>
           <t>Эфиопия Белойя гр.2</t>
         </is>
       </c>
-      <c r="C40" s="14" t="inlineStr">
+      <c r="C40" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D40" s="15" t="n">
+      <c r="D40" s="12" t="n">
         <v>2232.5</v>
       </c>
-      <c r="E40" s="15" t="n">
+      <c r="E40" s="12" t="n">
         <v>2010</v>
       </c>
-      <c r="F40" s="15" t="n">
+      <c r="F40" s="12" t="n">
         <v>1790</v>
       </c>
-      <c r="G40" s="15" t="n">
+      <c r="G40" s="12" t="n">
         <v>525</v>
       </c>
-      <c r="H40" s="15" t="n">
+      <c r="H40" s="12" t="n">
         <v>472.5</v>
       </c>
-      <c r="I40" s="15" t="n">
+      <c r="I40" s="12" t="n">
         <v>420</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="13" t="inlineStr">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
+      <c r="B41" s="10" t="inlineStr">
         <is>
           <t>Эфиопия Челелекту гр.1</t>
         </is>
       </c>
-      <c r="C41" s="14" t="inlineStr">
+      <c r="C41" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D41" s="15" t="n">
+      <c r="D41" s="12" t="n">
         <v>2862.5</v>
       </c>
-      <c r="E41" s="15" t="n">
+      <c r="E41" s="12" t="n">
         <v>2580</v>
       </c>
-      <c r="F41" s="15" t="n">
+      <c r="F41" s="12" t="n">
         <v>2290</v>
       </c>
-      <c r="G41" s="15" t="n">
+      <c r="G41" s="12" t="n">
         <v>655</v>
       </c>
-      <c r="H41" s="15" t="n">
+      <c r="H41" s="12" t="n">
         <v>589.5</v>
       </c>
-      <c r="I41" s="15" t="n">
+      <c r="I41" s="12" t="n">
         <v>525</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="13" t="inlineStr">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>микролот • BLACK</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
+      <c r="B42" s="10" t="inlineStr">
         <is>
           <t>Эфиопия Челчеле гр.1</t>
         </is>
       </c>
-      <c r="C42" s="14" t="inlineStr">
+      <c r="C42" s="11" t="inlineStr">
         <is>
           <t>E F</t>
         </is>
       </c>
-      <c r="D42" s="15" t="n">
+      <c r="D42" s="12" t="n">
         <v>2862.5</v>
       </c>
-      <c r="E42" s="15" t="n">
+      <c r="E42" s="12" t="n">
         <v>2580</v>
       </c>
-      <c r="F42" s="15" t="n">
+      <c r="F42" s="12" t="n">
         <v>2290</v>
       </c>
-      <c r="G42" s="15" t="n">
+      <c r="G42" s="12" t="n">
         <v>655</v>
       </c>
-      <c r="H42" s="15" t="n">
+      <c r="H42" s="12" t="n">
         <v>589.5</v>
       </c>
-      <c r="I42" s="15" t="n">
+      <c r="I42" s="12" t="n">
         <v>525</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="13" t="inlineStr">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
+      <c r="B43" s="10" t="inlineStr">
         <is>
           <t>Бразилия SL28</t>
         </is>
       </c>
-      <c r="C43" s="14" t="inlineStr">
+      <c r="C43" s="11" t="inlineStr">
         <is>
           <t>E F</t>
         </is>
       </c>
-      <c r="D43" s="15" t="n">
+      <c r="D43" s="12" t="n">
         <v>3500</v>
       </c>
-      <c r="E43" s="15" t="n">
+      <c r="E43" s="12" t="n">
         <v>3150</v>
       </c>
-      <c r="F43" s="15" t="n">
+      <c r="F43" s="12" t="n">
         <v>2800</v>
       </c>
-      <c r="G43" s="15" t="n">
+      <c r="G43" s="12" t="n">
         <v>780</v>
       </c>
-      <c r="H43" s="15" t="n">
+      <c r="H43" s="12" t="n">
         <v>702</v>
       </c>
-      <c r="I43" s="15" t="n">
+      <c r="I43" s="12" t="n">
         <v>625</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="13" t="inlineStr">
+      <c r="A44" s="10" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B44" s="13" t="inlineStr">
+      <c r="B44" s="10" t="inlineStr">
         <is>
           <t>Бразилия Судан Руме</t>
         </is>
       </c>
-      <c r="C44" s="14" t="inlineStr">
+      <c r="C44" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D44" s="15" t="n">
+      <c r="D44" s="12" t="n">
         <v>3500</v>
       </c>
-      <c r="E44" s="15" t="n">
+      <c r="E44" s="12" t="n">
         <v>3150</v>
       </c>
-      <c r="F44" s="15" t="n">
+      <c r="F44" s="12" t="n">
         <v>2800</v>
       </c>
-      <c r="G44" s="15" t="n">
+      <c r="G44" s="12" t="n">
         <v>780</v>
       </c>
-      <c r="H44" s="15" t="n">
+      <c r="H44" s="12" t="n">
         <v>702</v>
       </c>
-      <c r="I44" s="15" t="n">
+      <c r="I44" s="12" t="n">
         <v>625</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="13" t="inlineStr">
+      <c r="A45" s="10" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
+      <c r="B45" s="10" t="inlineStr">
         <is>
           <t>Бразилия Фазенда Лагуинья мундо</t>
         </is>
       </c>
-      <c r="C45" s="14" t="inlineStr">
+      <c r="C45" s="11" t="inlineStr">
         <is>
           <t>E F</t>
         </is>
       </c>
-      <c r="D45" s="15" t="n">
+      <c r="D45" s="12" t="n">
         <v>3500</v>
       </c>
-      <c r="E45" s="15" t="n">
+      <c r="E45" s="12" t="n">
         <v>3150</v>
       </c>
-      <c r="F45" s="15" t="n">
+      <c r="F45" s="12" t="n">
         <v>2800</v>
       </c>
-      <c r="G45" s="15" t="n">
+      <c r="G45" s="12" t="n">
         <v>780</v>
       </c>
-      <c r="H45" s="15" t="n">
+      <c r="H45" s="12" t="n">
         <v>702</v>
       </c>
-      <c r="I45" s="15" t="n">
+      <c r="I45" s="12" t="n">
         <v>625</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>NEW микролот • BORЩ</t>
+          <t>микролот • BORЩ</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
@@ -2079,213 +2079,283 @@
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="13" t="inlineStr">
+      <c r="A47" s="10" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
+      <c r="B47" s="10" t="inlineStr">
         <is>
           <t>Колумбия Гонзало Кармона</t>
         </is>
       </c>
-      <c r="C47" s="14" t="inlineStr">
+      <c r="C47" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D47" s="15" t="n">
+      <c r="D47" s="12" t="n">
         <v>3500</v>
       </c>
-      <c r="E47" s="15" t="n">
+      <c r="E47" s="12" t="n">
         <v>3150</v>
       </c>
-      <c r="F47" s="15" t="n">
+      <c r="F47" s="12" t="n">
         <v>2800</v>
       </c>
-      <c r="G47" s="15" t="n">
+      <c r="G47" s="12" t="n">
         <v>780</v>
       </c>
-      <c r="H47" s="15" t="n">
+      <c r="H47" s="12" t="n">
         <v>702</v>
       </c>
-      <c r="I47" s="15" t="n">
+      <c r="I47" s="12" t="n">
         <v>625</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="13" t="inlineStr">
+      <c r="A48" s="10" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B48" s="13" t="inlineStr">
+      <c r="B48" s="10" t="inlineStr">
         <is>
           <t>Колумбия Маракуйя</t>
         </is>
       </c>
-      <c r="C48" s="14" t="inlineStr">
+      <c r="C48" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D48" s="15" t="n">
+      <c r="D48" s="12" t="n">
         <v>5922.5</v>
       </c>
-      <c r="E48" s="15" t="n">
+      <c r="E48" s="12" t="n">
         <v>5335</v>
       </c>
-      <c r="F48" s="15" t="n">
+      <c r="F48" s="12" t="n">
         <v>4740</v>
       </c>
-      <c r="G48" s="15" t="n">
+      <c r="G48" s="12" t="n">
         <v>1265</v>
       </c>
-      <c r="H48" s="15" t="n">
+      <c r="H48" s="12" t="n">
         <v>1138.5</v>
       </c>
-      <c r="I48" s="15" t="n">
+      <c r="I48" s="12" t="n">
         <v>1015</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="13" t="inlineStr">
+      <c r="A49" s="10" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
+      <c r="B49" s="10" t="inlineStr">
         <is>
           <t>Колумбия Пачамама</t>
         </is>
       </c>
-      <c r="C49" s="14" t="inlineStr">
+      <c r="C49" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D49" s="15" t="n">
+      <c r="D49" s="12" t="n">
         <v>4842.5</v>
       </c>
-      <c r="E49" s="15" t="n">
+      <c r="E49" s="12" t="n">
         <v>4360</v>
       </c>
-      <c r="F49" s="15" t="n">
+      <c r="F49" s="12" t="n">
         <v>3875</v>
       </c>
-      <c r="G49" s="15" t="n">
+      <c r="G49" s="12" t="n">
         <v>1050</v>
       </c>
-      <c r="H49" s="15" t="n">
+      <c r="H49" s="12" t="n">
         <v>945</v>
       </c>
-      <c r="I49" s="15" t="n">
+      <c r="I49" s="12" t="n">
         <v>840</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="13" t="inlineStr">
+      <c r="A50" s="10" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
+      <c r="B50" s="10" t="inlineStr">
         <is>
           <t>Колумбия Хайро Арсила</t>
         </is>
       </c>
-      <c r="C50" s="14" t="inlineStr">
+      <c r="C50" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D50" s="15" t="n">
+      <c r="D50" s="12" t="n">
         <v>2862.5</v>
       </c>
-      <c r="E50" s="15" t="n">
+      <c r="E50" s="12" t="n">
         <v>2580</v>
       </c>
-      <c r="F50" s="15" t="n">
+      <c r="F50" s="12" t="n">
         <v>2290</v>
       </c>
-      <c r="G50" s="15" t="n">
+      <c r="G50" s="12" t="n">
         <v>655</v>
       </c>
-      <c r="H50" s="15" t="n">
+      <c r="H50" s="12" t="n">
         <v>589.5</v>
       </c>
-      <c r="I50" s="15" t="n">
+      <c r="I50" s="12" t="n">
         <v>525</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="13" t="inlineStr">
+      <c r="A51" s="10" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
+      <c r="B51" s="10" t="inlineStr">
         <is>
           <t>Экваториальный блэнд</t>
         </is>
       </c>
-      <c r="C51" s="14" t="inlineStr">
+      <c r="C51" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D51" s="15" t="n">
+      <c r="D51" s="12" t="n">
         <v>3020</v>
       </c>
-      <c r="E51" s="15" t="n">
+      <c r="E51" s="12" t="n">
         <v>2720</v>
       </c>
-      <c r="F51" s="15" t="n">
+      <c r="F51" s="12" t="n">
         <v>2420</v>
       </c>
-      <c r="G51" s="15" t="n">
+      <c r="G51" s="12" t="n">
         <v>685</v>
       </c>
-      <c r="H51" s="15" t="n">
+      <c r="H51" s="12" t="n">
         <v>616.5</v>
       </c>
-      <c r="I51" s="15" t="n">
+      <c r="I51" s="12" t="n">
         <v>550</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="13" t="inlineStr">
+      <c r="A52" s="10" t="inlineStr">
         <is>
           <t>микролот • BORЩ</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
+      <c r="B52" s="10" t="inlineStr">
         <is>
           <t>Эфиопия Арича гр.1</t>
         </is>
       </c>
-      <c r="C52" s="14" t="inlineStr">
+      <c r="C52" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D52" s="15" t="n">
+      <c r="D52" s="12" t="n">
         <v>3020</v>
       </c>
-      <c r="E52" s="15" t="n">
+      <c r="E52" s="12" t="n">
         <v>2720</v>
       </c>
-      <c r="F52" s="15" t="n">
+      <c r="F52" s="12" t="n">
         <v>2420</v>
       </c>
-      <c r="G52" s="15" t="n">
+      <c r="G52" s="12" t="n">
         <v>685</v>
       </c>
-      <c r="H52" s="15" t="n">
+      <c r="H52" s="12" t="n">
         <v>616.5</v>
       </c>
-      <c r="I52" s="15" t="n">
+      <c r="I52" s="12" t="n">
         <v>550</v>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>NEW микролот</t>
+        </is>
+      </c>
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>Колумбия Катимор</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D53" s="15" t="n">
+        <v>4602.5</v>
+      </c>
+      <c r="E53" s="15" t="n">
+        <v>4145</v>
+      </c>
+      <c r="F53" s="15" t="n">
+        <v>3685</v>
+      </c>
+      <c r="G53" s="15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H53" s="15" t="n">
+        <v>900</v>
+      </c>
+      <c r="I53" s="15" t="n">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>NEW микролот</t>
+        </is>
+      </c>
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>Колумбия Катуррон</t>
+        </is>
+      </c>
+      <c r="C54" s="14" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D54" s="15" t="n">
+        <v>4602.5</v>
+      </c>
+      <c r="E54" s="15" t="n">
+        <v>4145</v>
+      </c>
+      <c r="F54" s="15" t="n">
+        <v>3685</v>
+      </c>
+      <c r="G54" s="15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H54" s="15" t="n">
+        <v>900</v>
+      </c>
+      <c r="I54" s="15" t="n">
+        <v>800</v>
       </c>
     </row>
   </sheetData>

</xml_diff>